<commit_message>
Switch HSS drills, taper drills, end mills and tool bits to Dormer; add Dormer RFQ sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4c5Y1XBRj63SkdBZ73bUS
</commit_message>
<xml_diff>
--- a/quotes/PR-217-228/RFQ_PR217_PR228.xlsx
+++ b/quotes/PR-217-228/RFQ_PR217_PR228.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licota Dealer" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tool Importer" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Welding-Safety-Consumables" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dormer Dealer" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tool Importer" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Welding-Safety-Consumables" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -942,7 +943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H93"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -958,7 +959,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Zidane Corporation - Request for Quotation (Tool Importer)</t>
+          <t>Zidane Corporation - Request for Quotation (Dormer Dealer)</t>
         </is>
       </c>
     </row>
@@ -1013,19 +1014,19 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>STONE CUTTING DISC 4"</t>
+          <t>DRILL BIT 08 MM (Yato or any Good brand taiwan)</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Dormer A002</t>
         </is>
       </c>
       <c r="E5" s="5" t="n"/>
@@ -1035,19 +1036,19 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>2</v>
+        <v>73</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>STEEL NAIL 1-1/2" Taiwan</t>
+          <t>HSS COBALT DRILL SET 1-13MM 25 PCS</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Generic (Taiwan)</t>
+          <t>Dormer A095 (HSS-Co)</t>
         </is>
       </c>
       <c r="E6" s="5" t="n"/>
@@ -1057,11 +1058,11 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>3</v>
+        <v>74</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>MECHANICAL JACK 5 TON (Japan or Germany)</t>
+          <t>HSS DRILL BITS 1/16-1/2" 29 PCS SET</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
@@ -1069,7 +1070,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Masada (Japan)</t>
+          <t>Dormer A095 (A002 x29)</t>
         </is>
       </c>
       <c r="E7" s="5" t="n"/>
@@ -1079,19 +1080,19 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>4</v>
+        <v>75</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>DRILL BIT 08 MM (Yato or any Good brand taiwan)</t>
+          <t>HSS DRILL BIT 14MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Dormer A130</t>
         </is>
       </c>
       <c r="E8" s="5" t="n"/>
@@ -1101,11 +1102,11 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>5</v>
+        <v>76</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>MECHANICAL JACK 03 TONS (Japan or germany)</t>
+          <t>HSS DRILL BIT 15MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
@@ -1113,7 +1114,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Masada (Japan)</t>
+          <t>Dormer A130</t>
         </is>
       </c>
       <c r="E9" s="5" t="n"/>
@@ -1123,19 +1124,19 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>41</v>
+        <v>77</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>CORDLESS IMPACT WRENCH 350N (Bosch)</t>
+          <t>HSS DRILL BIT 15.5MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Bosch Professional GDS 18V-350</t>
+          <t>Dormer A130</t>
         </is>
       </c>
       <c r="E10" s="5" t="n"/>
@@ -1145,19 +1146,19 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>45</v>
+        <v>78</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>ROUNDE FILE 12"</t>
+          <t>HSS DRILL BIT 16MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Dormer A130</t>
         </is>
       </c>
       <c r="E11" s="5" t="n"/>
@@ -1167,11 +1168,11 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>52</v>
+        <v>79</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>MECHANICAL PULLER 3 ARMED 200X200</t>
+          <t>HSS DRILL BIT 16.5MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
@@ -1179,7 +1180,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Dormer A130</t>
         </is>
       </c>
       <c r="E12" s="5" t="n"/>
@@ -1189,19 +1190,19 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>53</v>
+        <v>80</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>MECHANICAL PULLER 3 ARMED 250X250</t>
+          <t>HSS DRILL BIT 17MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Dormer A130</t>
         </is>
       </c>
       <c r="E13" s="5" t="n"/>
@@ -1211,11 +1212,11 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>55</v>
+        <v>81</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>MANUAL GREASE GUN 5KG</t>
+          <t>HSS DRILL BIT 17.5MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
@@ -1223,7 +1224,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Dormer A130</t>
         </is>
       </c>
       <c r="E14" s="5" t="n"/>
@@ -1233,11 +1234,11 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>60</v>
+        <v>82</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>STEEL MEASURMENT TAPE 100M</t>
+          <t>HSS DRILL BIT 19MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
@@ -1245,7 +1246,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Dormer A130</t>
         </is>
       </c>
       <c r="E15" s="5" t="n"/>
@@ -1255,19 +1256,19 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>REVOLVING CENTRE MT4</t>
+          <t>HSS DRILL BIT 21MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Vertex (Taiwan)</t>
+          <t>Dormer A130</t>
         </is>
       </c>
       <c r="E16" s="5" t="n"/>
@@ -1277,19 +1278,19 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>67</v>
+        <v>84</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>REVOLVING CENTRE MT3</t>
+          <t>HSS DRILL BIT 25MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Vertex (Taiwan)</t>
+          <t>Dormer A130</t>
         </is>
       </c>
       <c r="E17" s="5" t="n"/>
@@ -1299,19 +1300,19 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>CIRCUMFERENCE TAPE (60-950) (D20-300)</t>
+          <t>HSS DRILL BIT 30MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Insize</t>
+          <t>Dormer A130</t>
         </is>
       </c>
       <c r="E18" s="5" t="n"/>
@@ -1321,11 +1322,11 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>CIRCUMFERENCE TAPE (940-2200) (D300-700)</t>
+          <t>HSS DRILL BIT 32MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C19" s="4" t="n">
@@ -1333,7 +1334,7 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Insize</t>
+          <t>Dormer A130</t>
         </is>
       </c>
       <c r="E19" s="5" t="n"/>
@@ -1343,19 +1344,19 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BITS 1/16-1/2" 29 PCS SET</t>
+          <t>HSS DRILL BIT 35MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Dormer A130</t>
         </is>
       </c>
       <c r="E20" s="5" t="n"/>
@@ -1365,15 +1366,15 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 14MM TAPER SHANK</t>
+          <t>TAP SET 1/2" BSPF LEFT HAND (Dormer)</t>
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
@@ -1387,15 +1388,15 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 15MM TAPER SHANK</t>
+          <t>TAP SET 1/2" BSPF RIGHT HAND</t>
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
@@ -1409,15 +1410,15 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 15.5MM TAPER SHANK</t>
+          <t>TAP SET 3/8" BSPF</t>
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
@@ -1431,15 +1432,15 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 16MM TAPER SHANK</t>
+          <t>TAP SET 1/4" BSPF</t>
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
@@ -1453,15 +1454,15 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 16.5MM TAPER SHANK</t>
+          <t>TAP SET 1/8" BSPF</t>
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
@@ -1475,15 +1476,15 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>80</v>
+        <v>179</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 17MM TAPER SHANK</t>
+          <t>TAP SET 1" BSPF LEFT HAND</t>
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
@@ -1497,15 +1498,15 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>81</v>
+        <v>180</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 17.5MM TAPER SHANK</t>
+          <t>TAP SET 1" BSPF RIGHT HAND</t>
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
@@ -1519,15 +1520,15 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>82</v>
+        <v>181</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 19MM TAPER SHANK</t>
+          <t>TAP SET 1-1/4" BSPF LEFT HAND</t>
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
@@ -1541,11 +1542,11 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>83</v>
+        <v>182</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 21MM TAPER SHANK</t>
+          <t>TAP SET 1-1/4" BSPF RIGHT HAND</t>
         </is>
       </c>
       <c r="C29" s="4" t="n">
@@ -1563,19 +1564,19 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>84</v>
+        <v>204</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 25MM TAPER SHANK</t>
+          <t>END MILL CUTTER SIZE 5MM</t>
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Dormer</t>
+          <t>Dormer C-series HSS-Co</t>
         </is>
       </c>
       <c r="E30" s="5" t="n"/>
@@ -1585,19 +1586,19 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>85</v>
+        <v>205</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 30MM TAPER SHANK</t>
+          <t>END MILL CUTTER SIZE 6MM</t>
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Dormer</t>
+          <t>Dormer C-series HSS-Co</t>
         </is>
       </c>
       <c r="E31" s="5" t="n"/>
@@ -1607,19 +1608,19 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>86</v>
+        <v>206</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 32MM TAPER SHANK</t>
+          <t>END MILL CUTTER SIZE 8MM</t>
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Dormer</t>
+          <t>Dormer C-series HSS-Co</t>
         </is>
       </c>
       <c r="E32" s="5" t="n"/>
@@ -1629,19 +1630,19 @@
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>87</v>
+        <v>207</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 35MM TAPER SHANK</t>
+          <t>END MILL CUTTER SIZE 10MM</t>
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Dormer</t>
+          <t>Dormer C-series HSS-Co</t>
         </is>
       </c>
       <c r="E33" s="5" t="n"/>
@@ -1651,19 +1652,19 @@
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>88</v>
+        <v>208</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>MORSE TAPER EXTENSION SOCKET SLEEVE ADAPT</t>
+          <t>END MILL CUTTER SIZE 12MM</t>
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Vertex (Taiwan)</t>
+          <t>Dormer C-series HSS-Co</t>
         </is>
       </c>
       <c r="E34" s="5" t="n"/>
@@ -1673,19 +1674,19 @@
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>89</v>
+        <v>209</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>MORSE TAPER EXTENSION SOCKET SLEEVE ADAPT</t>
+          <t>END MILL CUTTER SIZE 16MM</t>
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Vertex (Taiwan)</t>
+          <t>Dormer C-series HSS-Co</t>
         </is>
       </c>
       <c r="E35" s="5" t="n"/>
@@ -1695,11 +1696,11 @@
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
-        <v>90</v>
+        <v>210</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>MORSE TAPER EXTENSION SOCKET SLEEVE ADAPT</t>
+          <t>END MILL CUTTER SIZE 18MM</t>
         </is>
       </c>
       <c r="C36" s="4" t="n">
@@ -1707,7 +1708,7 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Vertex (Taiwan)</t>
+          <t>Dormer C-series HSS-Co</t>
         </is>
       </c>
       <c r="E36" s="5" t="n"/>
@@ -1717,19 +1718,19 @@
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
-        <v>91</v>
+        <v>211</v>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>DEAD CENTRE DIAMOND TIP M2</t>
+          <t>END MILL CUTTER SIZE 22MM</t>
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Vertex (Taiwan)</t>
+          <t>Dormer C-series HSS-Co</t>
         </is>
       </c>
       <c r="E37" s="5" t="n"/>
@@ -1739,19 +1740,19 @@
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
-        <v>92</v>
+        <v>212</v>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>DEAD CENTRE DIAMOND TIP M3</t>
+          <t>END MILL CUTTER SIZE 25MM</t>
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Vertex (Taiwan)</t>
+          <t>Dormer C-series HSS-Co</t>
         </is>
       </c>
       <c r="E38" s="5" t="n"/>
@@ -1761,19 +1762,19 @@
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
-        <v>96</v>
+        <v>225</v>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>VERNIER DEPTH GUAGE 250MM GRADUATION 0.02M</t>
+          <t>HSS TOOL 08X08X200MM</t>
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Insize</t>
+          <t>Dormer</t>
         </is>
       </c>
       <c r="E39" s="5" t="n"/>
@@ -1783,19 +1784,19 @@
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
-        <v>97</v>
+        <v>226</v>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>CORDLESS DRILL DRIVER 150NM Bosch</t>
+          <t>HSS TOOL 10MMX10MMX200MM</t>
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Bosch Professional</t>
+          <t>Dormer</t>
         </is>
       </c>
       <c r="E40" s="5" t="n"/>
@@ -1805,15 +1806,15 @@
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
-        <v>98</v>
+        <v>227</v>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>TAP SET 1/2" BSPF LEFT HAND (Dormer)</t>
+          <t>HSS TOOL 12MMX12MMX200MM</t>
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
@@ -1827,15 +1828,15 @@
     </row>
     <row r="42">
       <c r="A42" s="4" t="n">
-        <v>99</v>
+        <v>228</v>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>TAP SET 1/2" BSPF RIGHT HAND</t>
+          <t>HSS TOOL 16MMX16MMX200MM</t>
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
@@ -1849,15 +1850,15 @@
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
-        <v>100</v>
+        <v>229</v>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>TAP SET 3/8" BSPF</t>
+          <t>HSS PARTING OFF TOOL 1/8" X 3/4" X 8"</t>
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
@@ -1871,1103 +1872,25 @@
     </row>
     <row r="44">
       <c r="A44" s="4" t="n">
-        <v>101</v>
+        <v>240</v>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>TAP SET 1/4" BSPF</t>
+          <t>DRILL BIT 4MM</t>
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>3</v>
+        <v>50</v>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Dormer</t>
+          <t>Dormer A002</t>
         </is>
       </c>
       <c r="E44" s="5" t="n"/>
       <c r="F44" s="6" t="n"/>
       <c r="G44" s="5" t="n"/>
       <c r="H44" s="4" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="n">
-        <v>102</v>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>TAP SET 1/8" BSPF</t>
-        </is>
-      </c>
-      <c r="C45" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>Dormer</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="n"/>
-      <c r="F45" s="6" t="n"/>
-      <c r="G45" s="5" t="n"/>
-      <c r="H45" s="4" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="n">
-        <v>107</v>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>C-CLAMP 12"</t>
-        </is>
-      </c>
-      <c r="C46" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="n"/>
-      <c r="F46" s="6" t="n"/>
-      <c r="G46" s="5" t="n"/>
-      <c r="H46" s="4" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="n">
-        <v>109</v>
-      </c>
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>MAGNET SPIRIT LEVEL 12"</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="n"/>
-      <c r="F47" s="6" t="n"/>
-      <c r="G47" s="5" t="n"/>
-      <c r="H47" s="4" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="n">
-        <v>110</v>
-      </c>
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>CARBON STEEL RIGHT ANGLE 150MM</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>Insize</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="n"/>
-      <c r="F48" s="6" t="n"/>
-      <c r="G48" s="5" t="n"/>
-      <c r="H48" s="4" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="n">
-        <v>179</v>
-      </c>
-      <c r="B49" s="4" t="inlineStr">
-        <is>
-          <t>TAP SET 1" BSPF LEFT HAND</t>
-        </is>
-      </c>
-      <c r="C49" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" s="4" t="inlineStr">
-        <is>
-          <t>Dormer</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="n"/>
-      <c r="F49" s="6" t="n"/>
-      <c r="G49" s="5" t="n"/>
-      <c r="H49" s="4" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="n">
-        <v>180</v>
-      </c>
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>TAP SET 1" BSPF RIGHT HAND</t>
-        </is>
-      </c>
-      <c r="C50" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>Dormer</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="n"/>
-      <c r="F50" s="6" t="n"/>
-      <c r="G50" s="5" t="n"/>
-      <c r="H50" s="4" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="n">
-        <v>181</v>
-      </c>
-      <c r="B51" s="4" t="inlineStr">
-        <is>
-          <t>TAP SET 1-1/4" BSPF LEFT HAND</t>
-        </is>
-      </c>
-      <c r="C51" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>Dormer</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="n"/>
-      <c r="F51" s="6" t="n"/>
-      <c r="G51" s="5" t="n"/>
-      <c r="H51" s="4" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="4" t="n">
-        <v>182</v>
-      </c>
-      <c r="B52" s="4" t="inlineStr">
-        <is>
-          <t>TAP SET 1-1/4" BSPF RIGHT HAND</t>
-        </is>
-      </c>
-      <c r="C52" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>Dormer</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="n"/>
-      <c r="F52" s="6" t="n"/>
-      <c r="G52" s="5" t="n"/>
-      <c r="H52" s="4" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="4" t="n">
-        <v>183</v>
-      </c>
-      <c r="B53" s="4" t="inlineStr">
-        <is>
-          <t>TAP SET M6</t>
-        </is>
-      </c>
-      <c r="C53" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D53" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="n"/>
-      <c r="F53" s="6" t="n"/>
-      <c r="G53" s="5" t="n"/>
-      <c r="H53" s="4" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="4" t="n">
-        <v>184</v>
-      </c>
-      <c r="B54" s="4" t="inlineStr">
-        <is>
-          <t>TAP SET M8</t>
-        </is>
-      </c>
-      <c r="C54" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="n"/>
-      <c r="F54" s="6" t="n"/>
-      <c r="G54" s="5" t="n"/>
-      <c r="H54" s="4" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="4" t="n">
-        <v>185</v>
-      </c>
-      <c r="B55" s="4" t="inlineStr">
-        <is>
-          <t>TAP SET M10</t>
-        </is>
-      </c>
-      <c r="C55" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="n"/>
-      <c r="F55" s="6" t="n"/>
-      <c r="G55" s="5" t="n"/>
-      <c r="H55" s="4" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="4" t="n">
-        <v>186</v>
-      </c>
-      <c r="B56" s="4" t="inlineStr">
-        <is>
-          <t>TAP SET M12</t>
-        </is>
-      </c>
-      <c r="C56" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E56" s="5" t="n"/>
-      <c r="F56" s="6" t="n"/>
-      <c r="G56" s="5" t="n"/>
-      <c r="H56" s="4" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="4" t="n">
-        <v>187</v>
-      </c>
-      <c r="B57" s="4" t="inlineStr">
-        <is>
-          <t>TAP SET M16</t>
-        </is>
-      </c>
-      <c r="C57" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D57" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="n"/>
-      <c r="F57" s="6" t="n"/>
-      <c r="G57" s="5" t="n"/>
-      <c r="H57" s="4" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="4" t="n">
-        <v>188</v>
-      </c>
-      <c r="B58" s="4" t="inlineStr">
-        <is>
-          <t>TAP SET M18</t>
-        </is>
-      </c>
-      <c r="C58" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D58" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E58" s="5" t="n"/>
-      <c r="F58" s="6" t="n"/>
-      <c r="G58" s="5" t="n"/>
-      <c r="H58" s="4" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="4" t="n">
-        <v>189</v>
-      </c>
-      <c r="B59" s="4" t="inlineStr">
-        <is>
-          <t>TAP SET M20</t>
-        </is>
-      </c>
-      <c r="C59" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D59" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="n"/>
-      <c r="F59" s="6" t="n"/>
-      <c r="G59" s="5" t="n"/>
-      <c r="H59" s="4" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="4" t="n">
-        <v>190</v>
-      </c>
-      <c r="B60" s="4" t="inlineStr">
-        <is>
-          <t>TAP HANDLE</t>
-        </is>
-      </c>
-      <c r="C60" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D60" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E60" s="5" t="n"/>
-      <c r="F60" s="6" t="n"/>
-      <c r="G60" s="5" t="n"/>
-      <c r="H60" s="4" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="4" t="n">
-        <v>191</v>
-      </c>
-      <c r="B61" s="4" t="inlineStr">
-        <is>
-          <t>TAP HANDLE</t>
-        </is>
-      </c>
-      <c r="C61" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D61" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E61" s="5" t="n"/>
-      <c r="F61" s="6" t="n"/>
-      <c r="G61" s="5" t="n"/>
-      <c r="H61" s="4" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="4" t="n">
-        <v>192</v>
-      </c>
-      <c r="B62" s="4" t="inlineStr">
-        <is>
-          <t>INSIDE CALIPER 06"</t>
-        </is>
-      </c>
-      <c r="C62" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D62" s="4" t="inlineStr">
-        <is>
-          <t>Generic (Taiwan)</t>
-        </is>
-      </c>
-      <c r="E62" s="5" t="n"/>
-      <c r="F62" s="6" t="n"/>
-      <c r="G62" s="5" t="n"/>
-      <c r="H62" s="4" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="4" t="n">
-        <v>193</v>
-      </c>
-      <c r="B63" s="4" t="inlineStr">
-        <is>
-          <t>INSIDE CALIPER 20"</t>
-        </is>
-      </c>
-      <c r="C63" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D63" s="4" t="inlineStr">
-        <is>
-          <t>Generic (Taiwan)</t>
-        </is>
-      </c>
-      <c r="E63" s="5" t="n"/>
-      <c r="F63" s="6" t="n"/>
-      <c r="G63" s="5" t="n"/>
-      <c r="H63" s="4" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="4" t="n">
-        <v>194</v>
-      </c>
-      <c r="B64" s="4" t="inlineStr">
-        <is>
-          <t>OUTSIDE CALIPER 06"</t>
-        </is>
-      </c>
-      <c r="C64" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D64" s="4" t="inlineStr">
-        <is>
-          <t>Generic (Taiwan)</t>
-        </is>
-      </c>
-      <c r="E64" s="5" t="n"/>
-      <c r="F64" s="6" t="n"/>
-      <c r="G64" s="5" t="n"/>
-      <c r="H64" s="4" t="n"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="4" t="n">
-        <v>195</v>
-      </c>
-      <c r="B65" s="4" t="inlineStr">
-        <is>
-          <t>OUTSIDE CALIPER 20"</t>
-        </is>
-      </c>
-      <c r="C65" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D65" s="4" t="inlineStr">
-        <is>
-          <t>Generic (Taiwan)</t>
-        </is>
-      </c>
-      <c r="E65" s="5" t="n"/>
-      <c r="F65" s="6" t="n"/>
-      <c r="G65" s="5" t="n"/>
-      <c r="H65" s="4" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="4" t="n">
-        <v>196</v>
-      </c>
-      <c r="B66" s="4" t="inlineStr">
-        <is>
-          <t>RACHET TAP HANDLE</t>
-        </is>
-      </c>
-      <c r="C66" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D66" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E66" s="5" t="n"/>
-      <c r="F66" s="6" t="n"/>
-      <c r="G66" s="5" t="n"/>
-      <c r="H66" s="4" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="4" t="n">
-        <v>202</v>
-      </c>
-      <c r="B67" s="4" t="inlineStr">
-        <is>
-          <t>NEEDLE FILE (5PCS SET)</t>
-        </is>
-      </c>
-      <c r="C67" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D67" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E67" s="5" t="n"/>
-      <c r="F67" s="6" t="n"/>
-      <c r="G67" s="5" t="n"/>
-      <c r="H67" s="4" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="4" t="n">
-        <v>204</v>
-      </c>
-      <c r="B68" s="4" t="inlineStr">
-        <is>
-          <t>END MILL CUTTER SIZE 5MM</t>
-        </is>
-      </c>
-      <c r="C68" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="D68" s="4" t="inlineStr">
-        <is>
-          <t>YG-1</t>
-        </is>
-      </c>
-      <c r="E68" s="5" t="n"/>
-      <c r="F68" s="6" t="n"/>
-      <c r="G68" s="5" t="n"/>
-      <c r="H68" s="4" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="4" t="n">
-        <v>205</v>
-      </c>
-      <c r="B69" s="4" t="inlineStr">
-        <is>
-          <t>END MILL CUTTER SIZE 6MM</t>
-        </is>
-      </c>
-      <c r="C69" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="D69" s="4" t="inlineStr">
-        <is>
-          <t>YG-1</t>
-        </is>
-      </c>
-      <c r="E69" s="5" t="n"/>
-      <c r="F69" s="6" t="n"/>
-      <c r="G69" s="5" t="n"/>
-      <c r="H69" s="4" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="4" t="n">
-        <v>206</v>
-      </c>
-      <c r="B70" s="4" t="inlineStr">
-        <is>
-          <t>END MILL CUTTER SIZE 8MM</t>
-        </is>
-      </c>
-      <c r="C70" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="D70" s="4" t="inlineStr">
-        <is>
-          <t>YG-1</t>
-        </is>
-      </c>
-      <c r="E70" s="5" t="n"/>
-      <c r="F70" s="6" t="n"/>
-      <c r="G70" s="5" t="n"/>
-      <c r="H70" s="4" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="4" t="n">
-        <v>207</v>
-      </c>
-      <c r="B71" s="4" t="inlineStr">
-        <is>
-          <t>END MILL CUTTER SIZE 10MM</t>
-        </is>
-      </c>
-      <c r="C71" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="D71" s="4" t="inlineStr">
-        <is>
-          <t>YG-1</t>
-        </is>
-      </c>
-      <c r="E71" s="5" t="n"/>
-      <c r="F71" s="6" t="n"/>
-      <c r="G71" s="5" t="n"/>
-      <c r="H71" s="4" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="4" t="n">
-        <v>208</v>
-      </c>
-      <c r="B72" s="4" t="inlineStr">
-        <is>
-          <t>END MILL CUTTER SIZE 12MM</t>
-        </is>
-      </c>
-      <c r="C72" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D72" s="4" t="inlineStr">
-        <is>
-          <t>YG-1</t>
-        </is>
-      </c>
-      <c r="E72" s="5" t="n"/>
-      <c r="F72" s="6" t="n"/>
-      <c r="G72" s="5" t="n"/>
-      <c r="H72" s="4" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="4" t="n">
-        <v>209</v>
-      </c>
-      <c r="B73" s="4" t="inlineStr">
-        <is>
-          <t>END MILL CUTTER SIZE 16MM</t>
-        </is>
-      </c>
-      <c r="C73" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D73" s="4" t="inlineStr">
-        <is>
-          <t>YG-1</t>
-        </is>
-      </c>
-      <c r="E73" s="5" t="n"/>
-      <c r="F73" s="6" t="n"/>
-      <c r="G73" s="5" t="n"/>
-      <c r="H73" s="4" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="4" t="n">
-        <v>210</v>
-      </c>
-      <c r="B74" s="4" t="inlineStr">
-        <is>
-          <t>END MILL CUTTER SIZE 18MM</t>
-        </is>
-      </c>
-      <c r="C74" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D74" s="4" t="inlineStr">
-        <is>
-          <t>YG-1</t>
-        </is>
-      </c>
-      <c r="E74" s="5" t="n"/>
-      <c r="F74" s="6" t="n"/>
-      <c r="G74" s="5" t="n"/>
-      <c r="H74" s="4" t="n"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="4" t="n">
-        <v>211</v>
-      </c>
-      <c r="B75" s="4" t="inlineStr">
-        <is>
-          <t>END MILL CUTTER SIZE 22MM</t>
-        </is>
-      </c>
-      <c r="C75" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D75" s="4" t="inlineStr">
-        <is>
-          <t>YG-1</t>
-        </is>
-      </c>
-      <c r="E75" s="5" t="n"/>
-      <c r="F75" s="6" t="n"/>
-      <c r="G75" s="5" t="n"/>
-      <c r="H75" s="4" t="n"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="4" t="n">
-        <v>212</v>
-      </c>
-      <c r="B76" s="4" t="inlineStr">
-        <is>
-          <t>END MILL CUTTER SIZE 25MM</t>
-        </is>
-      </c>
-      <c r="C76" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D76" s="4" t="inlineStr">
-        <is>
-          <t>YG-1</t>
-        </is>
-      </c>
-      <c r="E76" s="5" t="n"/>
-      <c r="F76" s="6" t="n"/>
-      <c r="G76" s="5" t="n"/>
-      <c r="H76" s="4" t="n"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="4" t="n">
-        <v>213</v>
-      </c>
-      <c r="B77" s="4" t="inlineStr">
-        <is>
-          <t>DIE NUT SIZE 5MM</t>
-        </is>
-      </c>
-      <c r="C77" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D77" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E77" s="5" t="n"/>
-      <c r="F77" s="6" t="n"/>
-      <c r="G77" s="5" t="n"/>
-      <c r="H77" s="4" t="n"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="4" t="n">
-        <v>214</v>
-      </c>
-      <c r="B78" s="4" t="inlineStr">
-        <is>
-          <t>DIE NUT SIZE 6MM</t>
-        </is>
-      </c>
-      <c r="C78" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D78" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E78" s="5" t="n"/>
-      <c r="F78" s="6" t="n"/>
-      <c r="G78" s="5" t="n"/>
-      <c r="H78" s="4" t="n"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="4" t="n">
-        <v>215</v>
-      </c>
-      <c r="B79" s="4" t="inlineStr">
-        <is>
-          <t>DIE NUT SIZE 8MM</t>
-        </is>
-      </c>
-      <c r="C79" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D79" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E79" s="5" t="n"/>
-      <c r="F79" s="6" t="n"/>
-      <c r="G79" s="5" t="n"/>
-      <c r="H79" s="4" t="n"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="4" t="n">
-        <v>216</v>
-      </c>
-      <c r="B80" s="4" t="inlineStr">
-        <is>
-          <t>DIE NUT SIZE 10MM</t>
-        </is>
-      </c>
-      <c r="C80" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D80" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E80" s="5" t="n"/>
-      <c r="F80" s="6" t="n"/>
-      <c r="G80" s="5" t="n"/>
-      <c r="H80" s="4" t="n"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="4" t="n">
-        <v>217</v>
-      </c>
-      <c r="B81" s="4" t="inlineStr">
-        <is>
-          <t>DIE NUT SIZE 12MM</t>
-        </is>
-      </c>
-      <c r="C81" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D81" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E81" s="5" t="n"/>
-      <c r="F81" s="6" t="n"/>
-      <c r="G81" s="5" t="n"/>
-      <c r="H81" s="4" t="n"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="4" t="n">
-        <v>218</v>
-      </c>
-      <c r="B82" s="4" t="inlineStr">
-        <is>
-          <t>DIE NUT SIZE 16MM</t>
-        </is>
-      </c>
-      <c r="C82" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D82" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E82" s="5" t="n"/>
-      <c r="F82" s="6" t="n"/>
-      <c r="G82" s="5" t="n"/>
-      <c r="H82" s="4" t="n"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="4" t="n">
-        <v>219</v>
-      </c>
-      <c r="B83" s="4" t="inlineStr">
-        <is>
-          <t>DIE NUT HANDLE SMALL</t>
-        </is>
-      </c>
-      <c r="C83" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D83" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E83" s="5" t="n"/>
-      <c r="F83" s="6" t="n"/>
-      <c r="G83" s="5" t="n"/>
-      <c r="H83" s="4" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="4" t="n">
-        <v>220</v>
-      </c>
-      <c r="B84" s="4" t="inlineStr">
-        <is>
-          <t>DIE NUT HANDLE MEDIUM</t>
-        </is>
-      </c>
-      <c r="C84" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D84" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E84" s="5" t="n"/>
-      <c r="F84" s="6" t="n"/>
-      <c r="G84" s="5" t="n"/>
-      <c r="H84" s="4" t="n"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="4" t="n">
-        <v>221</v>
-      </c>
-      <c r="B85" s="4" t="inlineStr">
-        <is>
-          <t>DIE NUT HANDLE LARGE</t>
-        </is>
-      </c>
-      <c r="C85" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D85" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E85" s="5" t="n"/>
-      <c r="F85" s="6" t="n"/>
-      <c r="G85" s="5" t="n"/>
-      <c r="H85" s="4" t="n"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="4" t="n">
-        <v>222</v>
-      </c>
-      <c r="B86" s="4" t="inlineStr">
-        <is>
-          <t>3 JAW CHUCK 4"</t>
-        </is>
-      </c>
-      <c r="C86" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D86" s="4" t="inlineStr">
-        <is>
-          <t>Vertex (Taiwan)</t>
-        </is>
-      </c>
-      <c r="E86" s="5" t="n"/>
-      <c r="F86" s="6" t="n"/>
-      <c r="G86" s="5" t="n"/>
-      <c r="H86" s="4" t="n"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="4" t="n">
-        <v>224</v>
-      </c>
-      <c r="B87" s="4" t="inlineStr">
-        <is>
-          <t>BENCH VISE 12"</t>
-        </is>
-      </c>
-      <c r="C87" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D87" s="4" t="inlineStr">
-        <is>
-          <t>Yato (heavy)</t>
-        </is>
-      </c>
-      <c r="E87" s="5" t="n"/>
-      <c r="F87" s="6" t="n"/>
-      <c r="G87" s="5" t="n"/>
-      <c r="H87" s="4" t="n"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="4" t="n">
-        <v>225</v>
-      </c>
-      <c r="B88" s="4" t="inlineStr">
-        <is>
-          <t>HSS TOOL 08X08X200MM</t>
-        </is>
-      </c>
-      <c r="C88" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="D88" s="4" t="inlineStr">
-        <is>
-          <t>Taiwan HSS</t>
-        </is>
-      </c>
-      <c r="E88" s="5" t="n"/>
-      <c r="F88" s="6" t="n"/>
-      <c r="G88" s="5" t="n"/>
-      <c r="H88" s="4" t="n"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="4" t="n">
-        <v>226</v>
-      </c>
-      <c r="B89" s="4" t="inlineStr">
-        <is>
-          <t>HSS TOOL 10MMX10MMX200MM</t>
-        </is>
-      </c>
-      <c r="C89" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="D89" s="4" t="inlineStr">
-        <is>
-          <t>Taiwan HSS</t>
-        </is>
-      </c>
-      <c r="E89" s="5" t="n"/>
-      <c r="F89" s="6" t="n"/>
-      <c r="G89" s="5" t="n"/>
-      <c r="H89" s="4" t="n"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="4" t="n">
-        <v>227</v>
-      </c>
-      <c r="B90" s="4" t="inlineStr">
-        <is>
-          <t>HSS TOOL 12MMX12MMX200MM</t>
-        </is>
-      </c>
-      <c r="C90" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="D90" s="4" t="inlineStr">
-        <is>
-          <t>Taiwan HSS</t>
-        </is>
-      </c>
-      <c r="E90" s="5" t="n"/>
-      <c r="F90" s="6" t="n"/>
-      <c r="G90" s="5" t="n"/>
-      <c r="H90" s="4" t="n"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="4" t="n">
-        <v>228</v>
-      </c>
-      <c r="B91" s="4" t="inlineStr">
-        <is>
-          <t>HSS TOOL 16MMX16MMX200MM</t>
-        </is>
-      </c>
-      <c r="C91" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="D91" s="4" t="inlineStr">
-        <is>
-          <t>Taiwan HSS</t>
-        </is>
-      </c>
-      <c r="E91" s="5" t="n"/>
-      <c r="F91" s="6" t="n"/>
-      <c r="G91" s="5" t="n"/>
-      <c r="H91" s="4" t="n"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="4" t="n">
-        <v>229</v>
-      </c>
-      <c r="B92" s="4" t="inlineStr">
-        <is>
-          <t>HSS PARTING OFF TOOL 1/8" X 3/4" X 8"</t>
-        </is>
-      </c>
-      <c r="C92" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="D92" s="4" t="inlineStr">
-        <is>
-          <t>Taiwan HSS</t>
-        </is>
-      </c>
-      <c r="E92" s="5" t="n"/>
-      <c r="F92" s="6" t="n"/>
-      <c r="G92" s="5" t="n"/>
-      <c r="H92" s="4" t="n"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="4" t="n">
-        <v>240</v>
-      </c>
-      <c r="B93" s="4" t="inlineStr">
-        <is>
-          <t>DRILL BIT 4MM</t>
-        </is>
-      </c>
-      <c r="C93" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D93" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E93" s="5" t="n"/>
-      <c r="F93" s="6" t="n"/>
-      <c r="G93" s="5" t="n"/>
-      <c r="H93" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2996,7 +1919,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Zidane Corporation - Request for Quotation (Welding-Safety-Consumables)</t>
+          <t>Zidane Corporation - Request for Quotation (Tool Importer)</t>
         </is>
       </c>
     </row>
@@ -3051,19 +1974,19 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>7 DRAWER TOOL TROLLEY</t>
+          <t>STONE CUTTING DISC 4"</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Bosch</t>
         </is>
       </c>
       <c r="E5" s="5" t="n"/>
@@ -3073,19 +1996,19 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>HOLLOW PUNCH (3MM-25MM) (15PCS SET)</t>
+          <t>STEEL NAIL 1-1/2" Taiwan</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Harden</t>
+          <t>Generic (Taiwan)</t>
         </is>
       </c>
       <c r="E6" s="5" t="n"/>
@@ -3095,19 +2018,19 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>SLEDGE HAMMER 1 LBS WITH FIBREGLASS HANDLE</t>
+          <t>MECHANICAL JACK 5 TON (Japan or Germany)</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Masada (Japan)</t>
         </is>
       </c>
       <c r="E7" s="5" t="n"/>
@@ -3117,19 +2040,19 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>73</v>
+        <v>5</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>HSS COBALT DRILL SET 1-13MM 25 PCS</t>
+          <t>MECHANICAL JACK 03 TONS (Japan or germany)</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Ingco</t>
+          <t>Masada (Japan)</t>
         </is>
       </c>
       <c r="E8" s="5" t="n"/>
@@ -3139,19 +2062,19 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>103</v>
+        <v>41</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>WIRE BRUSH HEAVY DUTY 4/5 NROW</t>
+          <t>CORDLESS IMPACT WRENCH 350N (Bosch)</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Bosch Professional GDS 18V-350</t>
         </is>
       </c>
       <c r="E9" s="5" t="n"/>
@@ -3161,11 +2084,11 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>104</v>
+        <v>45</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>WELDING HELMET (FLIP FRONT)</t>
+          <t>ROUNDE FILE 12"</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
@@ -3173,7 +2096,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E10" s="5" t="n"/>
@@ -3183,19 +2106,19 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>111</v>
+        <v>52</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>CARBON STEEL RIGHT ANGLE 300MM</t>
+          <t>MECHANICAL PULLER 3 ARMED 200X200</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Harden</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E11" s="5" t="n"/>
@@ -3205,19 +2128,19 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>112</v>
+        <v>53</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>GAS CUTTING TORCH MEDIUM 6-50MM</t>
+          <t>MECHANICAL PULLER 3 ARMED 250X250</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Harris type</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E12" s="5" t="n"/>
@@ -3227,19 +2150,19 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>113</v>
+        <v>55</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>CUTTING TIPS/NOZZLES NO. 02 (6MM-12MM)</t>
+          <t>MANUAL GREASE GUN 5KG</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E13" s="5" t="n"/>
@@ -3249,19 +2172,19 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>114</v>
+        <v>60</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>CUTTING TIPS/NOZZLES NO. 03 (12MM-25)</t>
+          <t>STEEL MEASURMENT TAPE 100M</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E14" s="5" t="n"/>
@@ -3271,11 +2194,11 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>116</v>
+        <v>66</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>FUEL GAS REGULATOR 0-2.5 BAR</t>
+          <t>REVOLVING CENTRE MT4</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
@@ -3283,7 +2206,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Vertex (Taiwan)</t>
         </is>
       </c>
       <c r="E15" s="5" t="n"/>
@@ -3293,19 +2216,19 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>117</v>
+        <v>67</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>OXYGEN HOSE 08MM ID</t>
+          <t>REVOLVING CENTRE MT3</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Vertex (Taiwan)</t>
         </is>
       </c>
       <c r="E16" s="5" t="n"/>
@@ -3315,19 +2238,19 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>118</v>
+        <v>69</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>ACETYLENE GAS HOSE 08 ID</t>
+          <t>CIRCUMFERENCE TAPE (60-950) (D20-300)</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Insize</t>
         </is>
       </c>
       <c r="E17" s="5" t="n"/>
@@ -3337,19 +2260,19 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>119</v>
+        <v>70</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER KEY/SPANNER</t>
+          <t>CIRCUMFERENCE TAPE (940-2200) (D300-700)</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Insize</t>
         </is>
       </c>
       <c r="E18" s="5" t="n"/>
@@ -3359,19 +2282,19 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>120</v>
+        <v>88</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>TIP CLEANER FOR GAS WELDING TORCH</t>
+          <t>MORSE TAPER EXTENSION SOCKET SLEEVE ADAPT</t>
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Vertex (Taiwan)</t>
         </is>
       </c>
       <c r="E19" s="5" t="n"/>
@@ -3381,19 +2304,19 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>122</v>
+        <v>89</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>AC/DC SINGLE PHASE WELDING PLANT 300 AMP</t>
+          <t>MORSE TAPER EXTENSION SOCKET SLEEVE ADAPT</t>
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Industrial (AC/DC TIG 300A)</t>
+          <t>Vertex (Taiwan)</t>
         </is>
       </c>
       <c r="E20" s="5" t="n"/>
@@ -3403,11 +2326,11 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>123</v>
+        <v>90</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>TIG WELDING TORCH AIR-COOLED 5METER</t>
+          <t>MORSE TAPER EXTENSION SOCKET SLEEVE ADAPT</t>
         </is>
       </c>
       <c r="C21" s="4" t="n">
@@ -3415,7 +2338,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Vertex (Taiwan)</t>
         </is>
       </c>
       <c r="E21" s="5" t="n"/>
@@ -3425,11 +2348,11 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>124</v>
+        <v>91</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>TORCH HEAD ARGON WELDING</t>
+          <t>DEAD CENTRE DIAMOND TIP M2</t>
         </is>
       </c>
       <c r="C22" s="4" t="n">
@@ -3437,7 +2360,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Vertex (Taiwan)</t>
         </is>
       </c>
       <c r="E22" s="5" t="n"/>
@@ -3447,19 +2370,19 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>125</v>
+        <v>92</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>COLLECT OF ARGON 2.4MM</t>
+          <t>DEAD CENTRE DIAMOND TIP M3</t>
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Vertex (Taiwan)</t>
         </is>
       </c>
       <c r="E23" s="5" t="n"/>
@@ -3469,19 +2392,19 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>126</v>
+        <v>96</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>COLLECT BODY FOR ARGON 2.4MM</t>
+          <t>VERNIER DEPTH GUAGE 250MM GRADUATION 0.02M</t>
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Insize</t>
         </is>
       </c>
       <c r="E24" s="5" t="n"/>
@@ -3491,19 +2414,19 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>127</v>
+        <v>97</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>CERAMIC CUP NO.5</t>
+          <t>CORDLESS DRILL DRIVER 150NM Bosch</t>
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Bosch Professional</t>
         </is>
       </c>
       <c r="E25" s="5" t="n"/>
@@ -3513,11 +2436,11 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>128</v>
+        <v>107</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>CERAMIC CUP NO.6</t>
+          <t>C-CLAMP 12"</t>
         </is>
       </c>
       <c r="C26" s="4" t="n">
@@ -3525,7 +2448,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E26" s="5" t="n"/>
@@ -3535,11 +2458,11 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>129</v>
+        <v>109</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>CERAMIC CUP NO.7</t>
+          <t>MAGNET SPIRIT LEVEL 12"</t>
         </is>
       </c>
       <c r="C27" s="4" t="n">
@@ -3547,7 +2470,7 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E27" s="5" t="n"/>
@@ -3557,19 +2480,19 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>TUNGSTEN ELECTRODE 2.4MM</t>
+          <t>CARBON STEEL RIGHT ANGLE 150MM</t>
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Insize</t>
         </is>
       </c>
       <c r="E28" s="5" t="n"/>
@@ -3579,19 +2502,19 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>132</v>
+        <v>183</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>ARGON GAS HOSE 06MM</t>
+          <t>TAP SET M6</t>
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E29" s="5" t="n"/>
@@ -3601,19 +2524,19 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>133</v>
+        <v>184</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>GAS HOSE CONNECTOR</t>
+          <t>TAP SET M8</t>
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E30" s="5" t="n"/>
@@ -3623,19 +2546,19 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>134</v>
+        <v>185</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>SHORT SLEEVE TIG WELDING GLOVES 10-INCH</t>
+          <t>TAP SET M10</t>
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E31" s="5" t="n"/>
@@ -3645,19 +2568,19 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>139</v>
+        <v>186</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>BUFFING DISC 125MM</t>
+          <t>TAP SET M12</t>
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E32" s="5" t="n"/>
@@ -3667,19 +2590,19 @@
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>140</v>
+        <v>187</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>BRASS PLATED CUP WIRE BRUSH 125MM</t>
+          <t>TAP SET M16</t>
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E33" s="5" t="n"/>
@@ -3689,19 +2612,19 @@
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>142</v>
+        <v>188</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>GRINDER WHEEL ALUMINIUM OXIDE GRIT 24</t>
+          <t>TAP SET M18</t>
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Norton</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E34" s="5" t="n"/>
@@ -3711,19 +2634,19 @@
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>143</v>
+        <v>189</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>GRINDER WHEEL ALUMINIUM OXIDE GRIT 60</t>
+          <t>TAP SET M20</t>
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Norton</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E35" s="5" t="n"/>
@@ -3733,19 +2656,19 @@
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
-        <v>144</v>
+        <v>190</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>GRINDER WHEEL SILICON CARBIDE</t>
+          <t>TAP HANDLE</t>
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Norton</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E36" s="5" t="n"/>
@@ -3755,19 +2678,19 @@
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
-        <v>145</v>
+        <v>191</v>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>COTTON ROPE 2MM</t>
+          <t>TAP HANDLE</t>
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>500</v>
+        <v>2</v>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E37" s="5" t="n"/>
@@ -3777,19 +2700,19 @@
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
-        <v>154</v>
+        <v>192</v>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>RED OXIDE POWDER</t>
+          <t>INSIDE CALIPER 06"</t>
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Generic (Taiwan)</t>
         </is>
       </c>
       <c r="E38" s="5" t="n"/>
@@ -3799,19 +2722,19 @@
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
-        <v>158</v>
+        <v>193</v>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>TOILET CLEANING BRUSH</t>
+          <t>INSIDE CALIPER 20"</t>
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Generic (Taiwan)</t>
         </is>
       </c>
       <c r="E39" s="5" t="n"/>
@@ -3821,19 +2744,19 @@
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
-        <v>159</v>
+        <v>194</v>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>CUT PIECES OF CLOTHS FOR CLEANING</t>
+          <t>OUTSIDE CALIPER 06"</t>
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Generic (Taiwan)</t>
         </is>
       </c>
       <c r="E40" s="5" t="n"/>
@@ -3843,19 +2766,19 @@
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
-        <v>160</v>
+        <v>195</v>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>ANCHOR BOLT 10X110</t>
+          <t>OUTSIDE CALIPER 20"</t>
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>150</v>
+        <v>2</v>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Generic (Taiwan)</t>
         </is>
       </c>
       <c r="E41" s="5" t="n"/>
@@ -3865,19 +2788,19 @@
     </row>
     <row r="42">
       <c r="A42" s="4" t="n">
-        <v>161</v>
+        <v>196</v>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>ANCHOR BOLT 12X120</t>
+          <t>RACHET TAP HANDLE</t>
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>150</v>
+        <v>2</v>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E42" s="5" t="n"/>
@@ -3887,19 +2810,19 @@
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
-        <v>162</v>
+        <v>202</v>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>ANCHOR BOLT 12X160</t>
+          <t>NEEDLE FILE (5PCS SET)</t>
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>150</v>
+        <v>2</v>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E43" s="5" t="n"/>
@@ -3909,19 +2832,19 @@
     </row>
     <row r="44">
       <c r="A44" s="4" t="n">
-        <v>164</v>
+        <v>213</v>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>WELDING RODS 2.5MM E6013, NO 10 Zodian</t>
+          <t>DIE NUT SIZE 5MM</t>
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Zodian</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E44" s="5" t="n"/>
@@ -3931,19 +2854,19 @@
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
-        <v>165</v>
+        <v>214</v>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>WELDING RODS 3.25MM E6013 NO 12</t>
+          <t>DIE NUT SIZE 6MM</t>
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Zodian</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E45" s="5" t="n"/>
@@ -3953,19 +2876,19 @@
     </row>
     <row r="46">
       <c r="A46" s="4" t="n">
-        <v>166</v>
+        <v>215</v>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>WELDING RODS 2.5MM E7018 NO-10</t>
+          <t>DIE NUT SIZE 8MM</t>
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Fortrex</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E46" s="5" t="n"/>
@@ -3975,19 +2898,19 @@
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
-        <v>167</v>
+        <v>216</v>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>SS WELDING RODS 309L-16 2.6MM NO.12</t>
+          <t>DIE NUT SIZE 10MM</t>
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E47" s="5" t="n"/>
@@ -3997,19 +2920,19 @@
     </row>
     <row r="48">
       <c r="A48" s="4" t="n">
-        <v>168</v>
+        <v>217</v>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>SS WELDING RODS 316L-16 2.6MM NO.12</t>
+          <t>DIE NUT SIZE 12MM</t>
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E48" s="5" t="n"/>
@@ -4019,19 +2942,19 @@
     </row>
     <row r="49">
       <c r="A49" s="4" t="n">
-        <v>177</v>
+        <v>218</v>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>BLIND RIVETS 04MMX25MM (1000PCS)</t>
+          <t>DIE NUT SIZE 16MM</t>
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Generic</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E49" s="5" t="n"/>
@@ -4041,11 +2964,11 @@
     </row>
     <row r="50">
       <c r="A50" s="4" t="n">
-        <v>230</v>
+        <v>219</v>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>HYDRAULIC JACK 3 TON</t>
+          <t>DIE NUT HANDLE SMALL</t>
         </is>
       </c>
       <c r="C50" s="4" t="n">
@@ -4053,7 +2976,7 @@
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Ronix</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E50" s="5" t="n"/>
@@ -4063,19 +2986,19 @@
     </row>
     <row r="51">
       <c r="A51" s="4" t="n">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>WELDING ELCTRODE HOLDER 1000 AMP</t>
+          <t>DIE NUT HANDLE MEDIUM</t>
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E51" s="5" t="n"/>
@@ -4085,19 +3008,19 @@
     </row>
     <row r="52">
       <c r="A52" s="4" t="n">
-        <v>235</v>
+        <v>221</v>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>EARTH CLAMP 1000 AMP</t>
+          <t>DIE NUT HANDLE LARGE</t>
         </is>
       </c>
       <c r="C52" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E52" s="5" t="n"/>
@@ -4107,19 +3030,19 @@
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
-        <v>236</v>
+        <v>222</v>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>WELDING CABLE 1000 AMPERE</t>
+          <t>3 JAW CHUCK 4"</t>
         </is>
       </c>
       <c r="C53" s="4" t="n">
-        <v>200</v>
+        <v>1</v>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Industrial (copper)</t>
+          <t>Vertex (Taiwan)</t>
         </is>
       </c>
       <c r="E53" s="5" t="n"/>
@@ -4129,19 +3052,19 @@
     </row>
     <row r="54">
       <c r="A54" s="4" t="n">
-        <v>237</v>
+        <v>224</v>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>CABLE LUGS 1000 AMPERE</t>
+          <t>BENCH VISE 12"</t>
         </is>
       </c>
       <c r="C54" s="4" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Yato (heavy)</t>
         </is>
       </c>
       <c r="E54" s="5" t="n"/>
@@ -4152,4 +3075,1162 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H53"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Zidane Corporation - Request for Quotation (Welding-Safety-Consumables)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Ref: PR-217 &amp; PR-228 | Please fill Unit Rate (PKR), brand offered and delivery time. Yellow cells = aap ne bharne hain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>SR#</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Item Description</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Preferred Brand</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Brand Offered</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Unit Rate (PKR)</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Delivery (days)</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>7 DRAWER TOOL TROLLEY</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>HOLLOW PUNCH (3MM-25MM) (15PCS SET)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Harden</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="4" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>SLEDGE HAMMER 1 LBS WITH FIBREGLASS HANDLE</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="4" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>103</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>WIRE BRUSH HEAVY DUTY 4/5 NROW</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="4" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>104</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>WELDING HELMET (FLIP FRONT)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="4" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>111</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>CARBON STEEL RIGHT ANGLE 300MM</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Harden</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="5" t="n"/>
+      <c r="H10" s="4" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>112</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>GAS CUTTING TORCH MEDIUM 6-50MM</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Harris type</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="5" t="n"/>
+      <c r="H11" s="4" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>113</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>CUTTING TIPS/NOZZLES NO. 02 (6MM-12MM)</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="5" t="n"/>
+      <c r="H12" s="4" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>114</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>CUTTING TIPS/NOZZLES NO. 03 (12MM-25)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="5" t="n"/>
+      <c r="H13" s="4" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>116</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>FUEL GAS REGULATOR 0-2.5 BAR</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="5" t="n"/>
+      <c r="H14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>117</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>OXYGEN HOSE 08MM ID</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="5" t="n"/>
+      <c r="H15" s="4" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>118</v>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>ACETYLENE GAS HOSE 08 ID</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="5" t="n"/>
+      <c r="H16" s="4" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>119</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>CYLINDER KEY/SPANNER</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="5" t="n"/>
+      <c r="H17" s="4" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>TIP CLEANER FOR GAS WELDING TORCH</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="5" t="n"/>
+      <c r="H18" s="4" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>122</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>AC/DC SINGLE PHASE WELDING PLANT 300 AMP</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Industrial (AC/DC TIG 300A)</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="5" t="n"/>
+      <c r="H19" s="4" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>123</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>TIG WELDING TORCH AIR-COOLED 5METER</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="5" t="n"/>
+      <c r="H20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>124</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>TORCH HEAD ARGON WELDING</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="5" t="n"/>
+      <c r="H21" s="4" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>125</v>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>COLLECT OF ARGON 2.4MM</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="5" t="n"/>
+      <c r="H22" s="4" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>126</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>COLLECT BODY FOR ARGON 2.4MM</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="6" t="n"/>
+      <c r="G23" s="5" t="n"/>
+      <c r="H23" s="4" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>127</v>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>CERAMIC CUP NO.5</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="n"/>
+      <c r="F24" s="6" t="n"/>
+      <c r="G24" s="5" t="n"/>
+      <c r="H24" s="4" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>128</v>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>CERAMIC CUP NO.6</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="n"/>
+      <c r="F25" s="6" t="n"/>
+      <c r="G25" s="5" t="n"/>
+      <c r="H25" s="4" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>129</v>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>CERAMIC CUP NO.7</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="n"/>
+      <c r="F26" s="6" t="n"/>
+      <c r="G26" s="5" t="n"/>
+      <c r="H26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>130</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>TUNGSTEN ELECTRODE 2.4MM</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="n"/>
+      <c r="F27" s="6" t="n"/>
+      <c r="G27" s="5" t="n"/>
+      <c r="H27" s="4" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>132</v>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>ARGON GAS HOSE 06MM</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="n"/>
+      <c r="F28" s="6" t="n"/>
+      <c r="G28" s="5" t="n"/>
+      <c r="H28" s="4" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>133</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>GAS HOSE CONNECTOR</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="n"/>
+      <c r="F29" s="6" t="n"/>
+      <c r="G29" s="5" t="n"/>
+      <c r="H29" s="4" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>134</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>SHORT SLEEVE TIG WELDING GLOVES 10-INCH</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="6" t="n"/>
+      <c r="G30" s="5" t="n"/>
+      <c r="H30" s="4" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>139</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>BUFFING DISC 125MM</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="n"/>
+      <c r="F31" s="6" t="n"/>
+      <c r="G31" s="5" t="n"/>
+      <c r="H31" s="4" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>140</v>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>BRASS PLATED CUP WIRE BRUSH 125MM</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="n"/>
+      <c r="F32" s="6" t="n"/>
+      <c r="G32" s="5" t="n"/>
+      <c r="H32" s="4" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>142</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>GRINDER WHEEL ALUMINIUM OXIDE GRIT 24</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Norton</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="n"/>
+      <c r="F33" s="6" t="n"/>
+      <c r="G33" s="5" t="n"/>
+      <c r="H33" s="4" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n">
+        <v>143</v>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>GRINDER WHEEL ALUMINIUM OXIDE GRIT 60</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Norton</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="n"/>
+      <c r="F34" s="6" t="n"/>
+      <c r="G34" s="5" t="n"/>
+      <c r="H34" s="4" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n">
+        <v>144</v>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>GRINDER WHEEL SILICON CARBIDE</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Norton</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="n"/>
+      <c r="F35" s="6" t="n"/>
+      <c r="G35" s="5" t="n"/>
+      <c r="H35" s="4" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n">
+        <v>145</v>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>COTTON ROPE 2MM</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="n">
+        <v>500</v>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="n"/>
+      <c r="F36" s="6" t="n"/>
+      <c r="G36" s="5" t="n"/>
+      <c r="H36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n">
+        <v>154</v>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>RED OXIDE POWDER</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="n"/>
+      <c r="F37" s="6" t="n"/>
+      <c r="G37" s="5" t="n"/>
+      <c r="H37" s="4" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="n">
+        <v>158</v>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>TOILET CLEANING BRUSH</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="n"/>
+      <c r="F38" s="6" t="n"/>
+      <c r="G38" s="5" t="n"/>
+      <c r="H38" s="4" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="n">
+        <v>159</v>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>CUT PIECES OF CLOTHS FOR CLEANING</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="n"/>
+      <c r="F39" s="6" t="n"/>
+      <c r="G39" s="5" t="n"/>
+      <c r="H39" s="4" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="n">
+        <v>160</v>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>ANCHOR BOLT 10X110</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="n"/>
+      <c r="F40" s="6" t="n"/>
+      <c r="G40" s="5" t="n"/>
+      <c r="H40" s="4" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n">
+        <v>161</v>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>ANCHOR BOLT 12X120</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="n"/>
+      <c r="F41" s="6" t="n"/>
+      <c r="G41" s="5" t="n"/>
+      <c r="H41" s="4" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="n">
+        <v>162</v>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>ANCHOR BOLT 12X160</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="n"/>
+      <c r="F42" s="6" t="n"/>
+      <c r="G42" s="5" t="n"/>
+      <c r="H42" s="4" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="n">
+        <v>164</v>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>WELDING RODS 2.5MM E6013, NO 10 Zodian</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Zodian</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="n"/>
+      <c r="F43" s="6" t="n"/>
+      <c r="G43" s="5" t="n"/>
+      <c r="H43" s="4" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="n">
+        <v>165</v>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>WELDING RODS 3.25MM E6013 NO 12</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Zodian</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="n"/>
+      <c r="F44" s="6" t="n"/>
+      <c r="G44" s="5" t="n"/>
+      <c r="H44" s="4" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="n">
+        <v>166</v>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>WELDING RODS 2.5MM E7018 NO-10</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Fortrex</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="n"/>
+      <c r="F45" s="6" t="n"/>
+      <c r="G45" s="5" t="n"/>
+      <c r="H45" s="4" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="n">
+        <v>167</v>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>SS WELDING RODS 309L-16 2.6MM NO.12</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="n"/>
+      <c r="F46" s="6" t="n"/>
+      <c r="G46" s="5" t="n"/>
+      <c r="H46" s="4" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="n">
+        <v>168</v>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>SS WELDING RODS 316L-16 2.6MM NO.12</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="n"/>
+      <c r="F47" s="6" t="n"/>
+      <c r="G47" s="5" t="n"/>
+      <c r="H47" s="4" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="n">
+        <v>177</v>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>BLIND RIVETS 04MMX25MM (1000PCS)</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="n"/>
+      <c r="F48" s="6" t="n"/>
+      <c r="G48" s="5" t="n"/>
+      <c r="H48" s="4" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="n">
+        <v>230</v>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>HYDRAULIC JACK 3 TON</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>Ronix</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="n"/>
+      <c r="F49" s="6" t="n"/>
+      <c r="G49" s="5" t="n"/>
+      <c r="H49" s="4" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="n">
+        <v>234</v>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>WELDING ELCTRODE HOLDER 1000 AMP</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="n"/>
+      <c r="F50" s="6" t="n"/>
+      <c r="G50" s="5" t="n"/>
+      <c r="H50" s="4" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="n">
+        <v>235</v>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>EARTH CLAMP 1000 AMP</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="n"/>
+      <c r="F51" s="6" t="n"/>
+      <c r="G51" s="5" t="n"/>
+      <c r="H51" s="4" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="n">
+        <v>236</v>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>WELDING CABLE 1000 AMPERE</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>Industrial (copper)</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="n"/>
+      <c r="F52" s="6" t="n"/>
+      <c r="G52" s="5" t="n"/>
+      <c r="H52" s="4" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="n">
+        <v>237</v>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>CABLE LUGS 1000 AMPERE</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="n"/>
+      <c r="F53" s="6" t="n"/>
+      <c r="G53" s="5" t="n"/>
+      <c r="H53" s="4" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Brand ladder: Licota first, then Yato, then quality brand; drop cheap substitutes, show Industrial for industrial lines
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4c5Y1XBRj63SkdBZ73bUS
</commit_message>
<xml_diff>
--- a/quotes/PR-217-228/RFQ_PR217_PR228.xlsx
+++ b/quotes/PR-217-228/RFQ_PR217_PR228.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -538,11 +538,11 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>DOUBLE OPEN END WRENCH 36X41</t>
+          <t>7 DRAWER TOOL TROLLEY</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
@@ -550,7 +550,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Licota</t>
+          <t>Licota (AWX series, empty)</t>
         </is>
       </c>
       <c r="E5" s="5" t="n"/>
@@ -560,15 +560,15 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>DOUBLE OPEN END WRENCH 41X46</t>
+          <t>DOUBLE OPEN RING OFFSET WRENCH SET (12PCS)</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
@@ -582,15 +582,15 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>ALLEN HEX KEY 12MM</t>
+          <t>DOUBLE OPEN END WRENCH 6 TO 32 (12 PCS SET)</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
@@ -604,11 +604,11 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>ALLEN (HEX) KEY 14MM</t>
+          <t>DOUBLE OPEN END WRENCH 36X41</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
@@ -626,11 +626,11 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>ALLEN (HEX) KEY 16MM</t>
+          <t>DOUBLE OPEN END WRENCH 41X46</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
@@ -648,11 +648,11 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>CIRCLIP PLIER INTERNAL STRAIGHT 230MM</t>
+          <t>COMBINATION WRENCH 8 TO 32 (14 PCS SET)</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
@@ -670,15 +670,15 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>CIRCLIP PLIER EXTERNAL STRAIGHT 230MM</t>
+          <t>HOLLOW PUNCH (3MM-25MM) (15PCS SET)</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
@@ -692,15 +692,15 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>VICE GRIP PLIER 08"</t>
+          <t>SHORT TYPE HEX KEY WRENCH SET (09PCS)</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
@@ -714,15 +714,15 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>HEX IMPACT ADAPTOR 1/2" FEMALE TO 1/4" FEMALE</t>
+          <t>ALLEN HEX KEY 12MM</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
@@ -736,11 +736,11 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>47</v>
+        <v>21</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>UNIVERSAL PULLER 2-ARMED WITH HOOK BRAKE 21</t>
+          <t>ALLEN (HEX) KEY 14MM</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
@@ -758,15 +758,15 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>UNIVERSAL PULLER 2-ARMED WITH HOOK BRAK 250</t>
+          <t>ALLEN (HEX) KEY 16MM</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
@@ -780,15 +780,15 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>UNIVERSAL PULLER 2-ARMED 160 X 300 MM 5T</t>
+          <t>CIRCLIP PLIER INTERNAL STRAIGHT 230MM</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
@@ -802,15 +802,15 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>UNIVERSAL PULLER 2-ARMED 250 X 300 MM 7.5T</t>
+          <t>CIRCLIP PLIER EXTERNAL STRAIGHT 230MM</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
@@ -824,15 +824,15 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>51</v>
+        <v>31</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>INTERNAL EXTRACTOR WITH REINFORCED COLLAR</t>
+          <t>PIPE WRENCH SIZE 10"</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
@@ -846,15 +846,15 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>56</v>
+        <v>32</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>AIR GREASE GUN 500CC</t>
+          <t>PIPE WRENCH SIZE 12"</t>
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
@@ -868,15 +868,15 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>58</v>
+        <v>34</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>GREASE PIPE 1/4"X12"</t>
+          <t>PIPE WRENCH SIZE 24"</t>
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
@@ -890,15 +890,15 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>59</v>
+        <v>35</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>DOUBLE HANDLE GREASE NOZZLE</t>
+          <t>PIPE WRENCH SIZE 36"</t>
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
@@ -912,11 +912,11 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>ALIGNING PRY BAR DIA 5/8" X 18" LENGTH</t>
+          <t>SLEDGE HAMMER 1 LBS WITH FIBREGLASS HANDLE</t>
         </is>
       </c>
       <c r="C22" s="4" t="n">
@@ -931,6 +931,380 @@
       <c r="F22" s="6" t="n"/>
       <c r="G22" s="5" t="n"/>
       <c r="H22" s="4" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>SLEDGE HAMMER 3 LBS WITH FIBREGLASS HANDLE</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Licota</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="6" t="n"/>
+      <c r="G23" s="5" t="n"/>
+      <c r="H23" s="4" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>SOFT FACE DEAD BLOW HAMMER 50MM</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Licota</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="n"/>
+      <c r="F24" s="6" t="n"/>
+      <c r="G24" s="5" t="n"/>
+      <c r="H24" s="4" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>VICE GRIP PLIER 08"</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Licota</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="n"/>
+      <c r="F25" s="6" t="n"/>
+      <c r="G25" s="5" t="n"/>
+      <c r="H25" s="4" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>HEX IMPACT ADAPTOR 1/2" FEMALE TO 1/4" FEMALE</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Licota</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="n"/>
+      <c r="F26" s="6" t="n"/>
+      <c r="G26" s="5" t="n"/>
+      <c r="H26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>UNIVERSAL PULLER 2-ARMED WITH HOOK BRAKE 21</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Licota</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="n"/>
+      <c r="F27" s="6" t="n"/>
+      <c r="G27" s="5" t="n"/>
+      <c r="H27" s="4" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>UNIVERSAL PULLER 2-ARMED WITH HOOK BRAK 250</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Licota</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="n"/>
+      <c r="F28" s="6" t="n"/>
+      <c r="G28" s="5" t="n"/>
+      <c r="H28" s="4" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>UNIVERSAL PULLER 2-ARMED 160 X 300 MM 5T</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Licota</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="n"/>
+      <c r="F29" s="6" t="n"/>
+      <c r="G29" s="5" t="n"/>
+      <c r="H29" s="4" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>UNIVERSAL PULLER 2-ARMED 250 X 300 MM 7.5T</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Licota</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="6" t="n"/>
+      <c r="G30" s="5" t="n"/>
+      <c r="H30" s="4" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>INTERNAL EXTRACTOR WITH REINFORCED COLLAR</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Licota</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="n"/>
+      <c r="F31" s="6" t="n"/>
+      <c r="G31" s="5" t="n"/>
+      <c r="H31" s="4" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>MECHANICAL PULLER 3 ARMED 200X200</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Licota</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="n"/>
+      <c r="F32" s="6" t="n"/>
+      <c r="G32" s="5" t="n"/>
+      <c r="H32" s="4" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>MECHANICAL PULLER 3 ARMED 250X250</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Licota</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="n"/>
+      <c r="F33" s="6" t="n"/>
+      <c r="G33" s="5" t="n"/>
+      <c r="H33" s="4" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>AIR GREASE GUN 500CC</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Licota</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="n"/>
+      <c r="F34" s="6" t="n"/>
+      <c r="G34" s="5" t="n"/>
+      <c r="H34" s="4" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n">
+        <v>58</v>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>GREASE PIPE 1/4"X12"</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Licota</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="n"/>
+      <c r="F35" s="6" t="n"/>
+      <c r="G35" s="5" t="n"/>
+      <c r="H35" s="4" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>DOUBLE HANDLE GREASE NOZZLE</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Licota</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="n"/>
+      <c r="F36" s="6" t="n"/>
+      <c r="G36" s="5" t="n"/>
+      <c r="H36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n">
+        <v>62</v>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>ALIGNING PRY BAR DIA 5/8" X 18" LENGTH</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Licota</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="n"/>
+      <c r="F37" s="6" t="n"/>
+      <c r="G37" s="5" t="n"/>
+      <c r="H37" s="4" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="n">
+        <v>63</v>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>ADJUSTABLE WRENCH 15"</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Licota</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="n"/>
+      <c r="F38" s="6" t="n"/>
+      <c r="G38" s="5" t="n"/>
+      <c r="H38" s="4" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="n">
+        <v>148</v>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>FLATE METAL SCRAPPER 50MM</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Licota</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="n"/>
+      <c r="F39" s="6" t="n"/>
+      <c r="G39" s="5" t="n"/>
+      <c r="H39" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1903,7 +2277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2106,11 +2480,11 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>MECHANICAL PULLER 3 ARMED 200X200</t>
+          <t>MANUAL GREASE GUN 5KG</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
@@ -2128,15 +2502,15 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>MECHANICAL PULLER 3 ARMED 250X250</t>
+          <t>STEEL MEASURMENT TAPE 100M</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
@@ -2150,11 +2524,11 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>MANUAL GREASE GUN 5KG</t>
+          <t>STEEL MEASURMENT TAPE 50M</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
@@ -2172,11 +2546,11 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>STEEL MEASURMENT TAPE 100M</t>
+          <t>REVOLVING CENTRE MT4</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
@@ -2184,7 +2558,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Vertex (Taiwan)</t>
         </is>
       </c>
       <c r="E14" s="5" t="n"/>
@@ -2194,11 +2568,11 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>REVOLVING CENTRE MT4</t>
+          <t>REVOLVING CENTRE MT3</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
@@ -2216,11 +2590,11 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>REVOLVING CENTRE MT3</t>
+          <t>CIRCUMFERENCE TAPE (60-950) (D20-300)</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
@@ -2228,7 +2602,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Vertex (Taiwan)</t>
+          <t>Insize</t>
         </is>
       </c>
       <c r="E16" s="5" t="n"/>
@@ -2238,15 +2612,15 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>CIRCUMFERENCE TAPE (60-950) (D20-300)</t>
+          <t>CIRCUMFERENCE TAPE (940-2200) (D300-700)</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
@@ -2260,11 +2634,11 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>CIRCUMFERENCE TAPE (940-2200) (D300-700)</t>
+          <t>MEASURING TAPE 5M</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
@@ -2272,7 +2646,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Insize</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E18" s="5" t="n"/>
@@ -2436,11 +2810,11 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>C-CLAMP 12"</t>
+          <t>C-CLAMP 6"</t>
         </is>
       </c>
       <c r="C26" s="4" t="n">
@@ -2458,11 +2832,11 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>MAGNET SPIRIT LEVEL 12"</t>
+          <t>C-CLAMP 12"</t>
         </is>
       </c>
       <c r="C27" s="4" t="n">
@@ -2480,11 +2854,11 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>CARBON STEEL RIGHT ANGLE 150MM</t>
+          <t>SPIRIT LEVEL 1 METER</t>
         </is>
       </c>
       <c r="C28" s="4" t="n">
@@ -2492,7 +2866,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Insize</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E28" s="5" t="n"/>
@@ -2502,15 +2876,15 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>183</v>
+        <v>109</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>TAP SET M6</t>
+          <t>MAGNET SPIRIT LEVEL 12"</t>
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
@@ -2524,11 +2898,11 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>184</v>
+        <v>110</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>TAP SET M8</t>
+          <t>CARBON STEEL RIGHT ANGLE 150MM</t>
         </is>
       </c>
       <c r="C30" s="4" t="n">
@@ -2536,7 +2910,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Insize</t>
         </is>
       </c>
       <c r="E30" s="5" t="n"/>
@@ -2546,11 +2920,11 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>185</v>
+        <v>111</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>TAP SET M10</t>
+          <t>CARBON STEEL RIGHT ANGLE 300MM</t>
         </is>
       </c>
       <c r="C31" s="4" t="n">
@@ -2558,7 +2932,7 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Insize</t>
         </is>
       </c>
       <c r="E31" s="5" t="n"/>
@@ -2568,11 +2942,11 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>TAP SET M12</t>
+          <t>TAP SET M6</t>
         </is>
       </c>
       <c r="C32" s="4" t="n">
@@ -2590,15 +2964,15 @@
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>TAP SET M16</t>
+          <t>TAP SET M8</t>
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
@@ -2612,15 +2986,15 @@
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>TAP SET M18</t>
+          <t>TAP SET M10</t>
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
@@ -2634,15 +3008,15 @@
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>TAP SET M20</t>
+          <t>TAP SET M12</t>
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
@@ -2656,11 +3030,11 @@
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>TAP HANDLE</t>
+          <t>TAP SET M16</t>
         </is>
       </c>
       <c r="C36" s="4" t="n">
@@ -2678,15 +3052,15 @@
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>TAP HANDLE</t>
+          <t>TAP SET M18</t>
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
@@ -2700,19 +3074,19 @@
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>INSIDE CALIPER 06"</t>
+          <t>TAP SET M20</t>
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Generic (Taiwan)</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E38" s="5" t="n"/>
@@ -2722,11 +3096,11 @@
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>INSIDE CALIPER 20"</t>
+          <t>TAP HANDLE</t>
         </is>
       </c>
       <c r="C39" s="4" t="n">
@@ -2734,7 +3108,7 @@
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Generic (Taiwan)</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E39" s="5" t="n"/>
@@ -2744,19 +3118,19 @@
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>OUTSIDE CALIPER 06"</t>
+          <t>TAP HANDLE</t>
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Generic (Taiwan)</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E40" s="5" t="n"/>
@@ -2766,15 +3140,15 @@
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>OUTSIDE CALIPER 20"</t>
+          <t>INSIDE CALIPER 06"</t>
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
@@ -2788,11 +3162,11 @@
     </row>
     <row r="42">
       <c r="A42" s="4" t="n">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>RACHET TAP HANDLE</t>
+          <t>INSIDE CALIPER 20"</t>
         </is>
       </c>
       <c r="C42" s="4" t="n">
@@ -2800,7 +3174,7 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Generic (Taiwan)</t>
         </is>
       </c>
       <c r="E42" s="5" t="n"/>
@@ -2810,19 +3184,19 @@
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>NEEDLE FILE (5PCS SET)</t>
+          <t>OUTSIDE CALIPER 06"</t>
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Generic (Taiwan)</t>
         </is>
       </c>
       <c r="E43" s="5" t="n"/>
@@ -2832,11 +3206,11 @@
     </row>
     <row r="44">
       <c r="A44" s="4" t="n">
-        <v>213</v>
+        <v>195</v>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>DIE NUT SIZE 5MM</t>
+          <t>OUTSIDE CALIPER 20"</t>
         </is>
       </c>
       <c r="C44" s="4" t="n">
@@ -2844,7 +3218,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Generic (Taiwan)</t>
         </is>
       </c>
       <c r="E44" s="5" t="n"/>
@@ -2854,11 +3228,11 @@
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
-        <v>214</v>
+        <v>196</v>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>DIE NUT SIZE 6MM</t>
+          <t>RACHET TAP HANDLE</t>
         </is>
       </c>
       <c r="C45" s="4" t="n">
@@ -2876,11 +3250,11 @@
     </row>
     <row r="46">
       <c r="A46" s="4" t="n">
-        <v>215</v>
+        <v>202</v>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>DIE NUT SIZE 8MM</t>
+          <t>NEEDLE FILE (5PCS SET)</t>
         </is>
       </c>
       <c r="C46" s="4" t="n">
@@ -2898,11 +3272,11 @@
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>DIE NUT SIZE 10MM</t>
+          <t>DIE NUT SIZE 5MM</t>
         </is>
       </c>
       <c r="C47" s="4" t="n">
@@ -2920,11 +3294,11 @@
     </row>
     <row r="48">
       <c r="A48" s="4" t="n">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>DIE NUT SIZE 12MM</t>
+          <t>DIE NUT SIZE 6MM</t>
         </is>
       </c>
       <c r="C48" s="4" t="n">
@@ -2942,11 +3316,11 @@
     </row>
     <row r="49">
       <c r="A49" s="4" t="n">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>DIE NUT SIZE 16MM</t>
+          <t>DIE NUT SIZE 8MM</t>
         </is>
       </c>
       <c r="C49" s="4" t="n">
@@ -2964,15 +3338,15 @@
     </row>
     <row r="50">
       <c r="A50" s="4" t="n">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>DIE NUT HANDLE SMALL</t>
+          <t>DIE NUT SIZE 10MM</t>
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
@@ -2986,15 +3360,15 @@
     </row>
     <row r="51">
       <c r="A51" s="4" t="n">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>DIE NUT HANDLE MEDIUM</t>
+          <t>DIE NUT SIZE 12MM</t>
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
@@ -3008,15 +3382,15 @@
     </row>
     <row r="52">
       <c r="A52" s="4" t="n">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>DIE NUT HANDLE LARGE</t>
+          <t>DIE NUT SIZE 16MM</t>
         </is>
       </c>
       <c r="C52" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
@@ -3030,11 +3404,11 @@
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>3 JAW CHUCK 4"</t>
+          <t>DIE NUT HANDLE SMALL</t>
         </is>
       </c>
       <c r="C53" s="4" t="n">
@@ -3042,7 +3416,7 @@
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Vertex (Taiwan)</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E53" s="5" t="n"/>
@@ -3052,25 +3426,157 @@
     </row>
     <row r="54">
       <c r="A54" s="4" t="n">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>BENCH VISE 12"</t>
+          <t>DIE NUT HANDLE MEDIUM</t>
         </is>
       </c>
       <c r="C54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>Yato (heavy)</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E54" s="5" t="n"/>
       <c r="F54" s="6" t="n"/>
       <c r="G54" s="5" t="n"/>
       <c r="H54" s="4" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="n">
+        <v>221</v>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>DIE NUT HANDLE LARGE</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>Yato</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="n"/>
+      <c r="F55" s="6" t="n"/>
+      <c r="G55" s="5" t="n"/>
+      <c r="H55" s="4" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="n">
+        <v>222</v>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>3 JAW CHUCK 4"</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>Vertex (Taiwan)</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="n"/>
+      <c r="F56" s="6" t="n"/>
+      <c r="G56" s="5" t="n"/>
+      <c r="H56" s="4" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="n">
+        <v>223</v>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>BENCH VISE 08"</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>Yato YT-65049</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="n"/>
+      <c r="F57" s="6" t="n"/>
+      <c r="G57" s="5" t="n"/>
+      <c r="H57" s="4" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="n">
+        <v>224</v>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>BENCH VISE 12"</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Yato (heavy)</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="n"/>
+      <c r="F58" s="6" t="n"/>
+      <c r="G58" s="5" t="n"/>
+      <c r="H58" s="4" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="n">
+        <v>230</v>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>HYDRAULIC JACK 3 TON</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>Yato YT-17001</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="n"/>
+      <c r="F59" s="6" t="n"/>
+      <c r="G59" s="5" t="n"/>
+      <c r="H59" s="4" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="n">
+        <v>231</v>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>HYDRAULIC JACK 5 TON</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>Yato YT-17002</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="n"/>
+      <c r="F60" s="6" t="n"/>
+      <c r="G60" s="5" t="n"/>
+      <c r="H60" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3083,7 +3589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3154,19 +3660,19 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>7 DRAWER TOOL TROLLEY</t>
+          <t>WIRE BRUSH HEAVY DUTY 4/5 NROW</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="E5" s="5" t="n"/>
@@ -3176,11 +3682,11 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>16</v>
+        <v>104</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>HOLLOW PUNCH (3MM-25MM) (15PCS SET)</t>
+          <t>WELDING HELMET (FLIP FRONT)</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
@@ -3188,7 +3694,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Harden</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="E6" s="5" t="n"/>
@@ -3198,19 +3704,19 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>36</v>
+        <v>112</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>SLEDGE HAMMER 1 LBS WITH FIBREGLASS HANDLE</t>
+          <t>GAS CUTTING TORCH MEDIUM 6-50MM</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Harris type</t>
         </is>
       </c>
       <c r="E7" s="5" t="n"/>
@@ -3220,15 +3726,15 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>WIRE BRUSH HEAVY DUTY 4/5 NROW</t>
+          <t>CUTTING TIPS/NOZZLES NO. 02 (6MM-12MM)</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
@@ -3242,15 +3748,15 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>WELDING HELMET (FLIP FRONT)</t>
+          <t>CUTTING TIPS/NOZZLES NO. 03 (12MM-25)</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
@@ -3264,19 +3770,19 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>CARBON STEEL RIGHT ANGLE 300MM</t>
+          <t>FUEL GAS REGULATOR 0-2.5 BAR</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Harden</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="E10" s="5" t="n"/>
@@ -3286,19 +3792,19 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>GAS CUTTING TORCH MEDIUM 6-50MM</t>
+          <t>OXYGEN HOSE 08MM ID</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Harris type</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="E11" s="5" t="n"/>
@@ -3308,15 +3814,15 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>CUTTING TIPS/NOZZLES NO. 02 (6MM-12MM)</t>
+          <t>ACETYLENE GAS HOSE 08 ID</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
@@ -3330,15 +3836,15 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>CUTTING TIPS/NOZZLES NO. 03 (12MM-25)</t>
+          <t>CYLINDER KEY/SPANNER</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
@@ -3352,15 +3858,15 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>FUEL GAS REGULATOR 0-2.5 BAR</t>
+          <t>TIP CLEANER FOR GAS WELDING TORCH</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
@@ -3374,19 +3880,19 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>OXYGEN HOSE 08MM ID</t>
+          <t>AC/DC SINGLE PHASE WELDING PLANT 300 AMP</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Industrial (AC/DC TIG 300A)</t>
         </is>
       </c>
       <c r="E15" s="5" t="n"/>
@@ -3396,15 +3902,15 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>ACETYLENE GAS HOSE 08 ID</t>
+          <t>TIG WELDING TORCH AIR-COOLED 5METER</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
@@ -3418,11 +3924,11 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER KEY/SPANNER</t>
+          <t>TORCH HEAD ARGON WELDING</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
@@ -3440,15 +3946,15 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>TIP CLEANER FOR GAS WELDING TORCH</t>
+          <t>COLLECT OF ARGON 2.4MM</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
@@ -3462,19 +3968,19 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>AC/DC SINGLE PHASE WELDING PLANT 300 AMP</t>
+          <t>COLLECT BODY FOR ARGON 2.4MM</t>
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Industrial (AC/DC TIG 300A)</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="E19" s="5" t="n"/>
@@ -3484,15 +3990,15 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>TIG WELDING TORCH AIR-COOLED 5METER</t>
+          <t>CERAMIC CUP NO.5</t>
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
@@ -3506,15 +4012,15 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>TORCH HEAD ARGON WELDING</t>
+          <t>CERAMIC CUP NO.6</t>
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
@@ -3528,15 +4034,15 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>COLLECT OF ARGON 2.4MM</t>
+          <t>CERAMIC CUP NO.7</t>
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
@@ -3550,15 +4056,15 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>COLLECT BODY FOR ARGON 2.4MM</t>
+          <t>TUNGSTEN ELECTRODE 2.4MM</t>
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
@@ -3572,15 +4078,15 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>CERAMIC CUP NO.5</t>
+          <t>ARGON GAS HOSE 06MM</t>
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
@@ -3594,11 +4100,11 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>CERAMIC CUP NO.6</t>
+          <t>GAS HOSE CONNECTOR</t>
         </is>
       </c>
       <c r="C25" s="4" t="n">
@@ -3616,11 +4122,11 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>CERAMIC CUP NO.7</t>
+          <t>SHORT SLEEVE TIG WELDING GLOVES 10-INCH</t>
         </is>
       </c>
       <c r="C26" s="4" t="n">
@@ -3638,15 +4144,15 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>TUNGSTEN ELECTRODE 2.4MM</t>
+          <t>BUFFING DISC 125MM</t>
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
@@ -3660,15 +4166,15 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>ARGON GAS HOSE 06MM</t>
+          <t>BRASS PLATED CUP WIRE BRUSH 125MM</t>
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
@@ -3682,19 +4188,19 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>GAS HOSE CONNECTOR</t>
+          <t>GRINDER WHEEL ALUMINIUM OXIDE GRIT 24</t>
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Norton</t>
         </is>
       </c>
       <c r="E29" s="5" t="n"/>
@@ -3704,19 +4210,19 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>SHORT SLEEVE TIG WELDING GLOVES 10-INCH</t>
+          <t>GRINDER WHEEL ALUMINIUM OXIDE GRIT 60</t>
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Norton</t>
         </is>
       </c>
       <c r="E30" s="5" t="n"/>
@@ -3726,19 +4232,19 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>BUFFING DISC 125MM</t>
+          <t>GRINDER WHEEL SILICON CARBIDE</t>
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Norton</t>
         </is>
       </c>
       <c r="E31" s="5" t="n"/>
@@ -3748,19 +4254,19 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>BRASS PLATED CUP WIRE BRUSH 125MM</t>
+          <t>COTTON ROPE 2MM</t>
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>24</v>
+        <v>500</v>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Local</t>
         </is>
       </c>
       <c r="E32" s="5" t="n"/>
@@ -3770,19 +4276,19 @@
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>GRINDER WHEEL ALUMINIUM OXIDE GRIT 24</t>
+          <t>RED OXIDE POWDER</t>
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Norton</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="E33" s="5" t="n"/>
@@ -3792,19 +4298,19 @@
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>143</v>
+        <v>158</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>GRINDER WHEEL ALUMINIUM OXIDE GRIT 60</t>
+          <t>TOILET CLEANING BRUSH</t>
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Norton</t>
+          <t>Local</t>
         </is>
       </c>
       <c r="E34" s="5" t="n"/>
@@ -3814,19 +4320,19 @@
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>144</v>
+        <v>159</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>GRINDER WHEEL SILICON CARBIDE</t>
+          <t>CUT PIECES OF CLOTHS FOR CLEANING</t>
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>3</v>
+        <v>100</v>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Norton</t>
+          <t>Local</t>
         </is>
       </c>
       <c r="E35" s="5" t="n"/>
@@ -3836,15 +4342,15 @@
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
-        <v>145</v>
+        <v>160</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>COTTON ROPE 2MM</t>
+          <t>ANCHOR BOLT 10X110</t>
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>500</v>
+        <v>150</v>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
@@ -3858,19 +4364,19 @@
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>RED OXIDE POWDER</t>
+          <t>ANCHOR BOLT 12X120</t>
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>12</v>
+        <v>150</v>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Local</t>
         </is>
       </c>
       <c r="E37" s="5" t="n"/>
@@ -3880,15 +4386,15 @@
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>TOILET CLEANING BRUSH</t>
+          <t>ANCHOR BOLT 12X160</t>
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>12</v>
+        <v>150</v>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
@@ -3902,19 +4408,19 @@
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>CUT PIECES OF CLOTHS FOR CLEANING</t>
+          <t>WELDING RODS 2.5MM E6013, NO 10 Zodian</t>
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Zodian</t>
         </is>
       </c>
       <c r="E39" s="5" t="n"/>
@@ -3924,19 +4430,19 @@
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>ANCHOR BOLT 10X110</t>
+          <t>WELDING RODS 3.25MM E6013 NO 12</t>
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>150</v>
+        <v>40</v>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Zodian</t>
         </is>
       </c>
       <c r="E40" s="5" t="n"/>
@@ -3946,19 +4452,19 @@
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>ANCHOR BOLT 12X120</t>
+          <t>WELDING RODS 2.5MM E7018 NO-10</t>
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>150</v>
+        <v>20</v>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Fortrex</t>
         </is>
       </c>
       <c r="E41" s="5" t="n"/>
@@ -3968,19 +4474,19 @@
     </row>
     <row r="42">
       <c r="A42" s="4" t="n">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>ANCHOR BOLT 12X160</t>
+          <t>SS WELDING RODS 309L-16 2.6MM NO.12</t>
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>150</v>
+        <v>40</v>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="E42" s="5" t="n"/>
@@ -3990,19 +4496,19 @@
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>WELDING RODS 2.5MM E6013, NO 10 Zodian</t>
+          <t>SS WELDING RODS 316L-16 2.6MM NO.12</t>
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Zodian</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="E43" s="5" t="n"/>
@@ -4012,19 +4518,19 @@
     </row>
     <row r="44">
       <c r="A44" s="4" t="n">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>WELDING RODS 3.25MM E6013 NO 12</t>
+          <t>BLIND RIVETS 04MMX25MM (1000PCS)</t>
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Zodian</t>
+          <t>Generic</t>
         </is>
       </c>
       <c r="E44" s="5" t="n"/>
@@ -4034,19 +4540,19 @@
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
-        <v>166</v>
+        <v>234</v>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>WELDING RODS 2.5MM E7018 NO-10</t>
+          <t>WELDING ELCTRODE HOLDER 1000 AMP</t>
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Fortrex</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E45" s="5" t="n"/>
@@ -4056,15 +4562,15 @@
     </row>
     <row r="46">
       <c r="A46" s="4" t="n">
-        <v>167</v>
+        <v>235</v>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>SS WELDING RODS 309L-16 2.6MM NO.12</t>
+          <t>EARTH CLAMP 1000 AMP</t>
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
@@ -4078,19 +4584,19 @@
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
-        <v>168</v>
+        <v>236</v>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>SS WELDING RODS 316L-16 2.6MM NO.12</t>
+          <t>WELDING CABLE 1000 AMPERE</t>
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>20</v>
+        <v>200</v>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Industrial (copper)</t>
         </is>
       </c>
       <c r="E47" s="5" t="n"/>
@@ -4100,19 +4606,19 @@
     </row>
     <row r="48">
       <c r="A48" s="4" t="n">
-        <v>177</v>
+        <v>237</v>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>BLIND RIVETS 04MMX25MM (1000PCS)</t>
+          <t>CABLE LUGS 1000 AMPERE</t>
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Generic</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="E48" s="5" t="n"/>
@@ -4120,116 +4626,6 @@
       <c r="G48" s="5" t="n"/>
       <c r="H48" s="4" t="n"/>
     </row>
-    <row r="49">
-      <c r="A49" s="4" t="n">
-        <v>230</v>
-      </c>
-      <c r="B49" s="4" t="inlineStr">
-        <is>
-          <t>HYDRAULIC JACK 3 TON</t>
-        </is>
-      </c>
-      <c r="C49" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" s="4" t="inlineStr">
-        <is>
-          <t>Ronix</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="n"/>
-      <c r="F49" s="6" t="n"/>
-      <c r="G49" s="5" t="n"/>
-      <c r="H49" s="4" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="n">
-        <v>234</v>
-      </c>
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>WELDING ELCTRODE HOLDER 1000 AMP</t>
-        </is>
-      </c>
-      <c r="C50" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="n"/>
-      <c r="F50" s="6" t="n"/>
-      <c r="G50" s="5" t="n"/>
-      <c r="H50" s="4" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="n">
-        <v>235</v>
-      </c>
-      <c r="B51" s="4" t="inlineStr">
-        <is>
-          <t>EARTH CLAMP 1000 AMP</t>
-        </is>
-      </c>
-      <c r="C51" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>Industrial</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="n"/>
-      <c r="F51" s="6" t="n"/>
-      <c r="G51" s="5" t="n"/>
-      <c r="H51" s="4" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="4" t="n">
-        <v>236</v>
-      </c>
-      <c r="B52" s="4" t="inlineStr">
-        <is>
-          <t>WELDING CABLE 1000 AMPERE</t>
-        </is>
-      </c>
-      <c r="C52" s="4" t="n">
-        <v>200</v>
-      </c>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>Industrial (copper)</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="n"/>
-      <c r="F52" s="6" t="n"/>
-      <c r="G52" s="5" t="n"/>
-      <c r="H52" s="4" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="4" t="n">
-        <v>237</v>
-      </c>
-      <c r="B53" s="4" t="inlineStr">
-        <is>
-          <t>CABLE LUGS 1000 AMPERE</t>
-        </is>
-      </c>
-      <c r="C53" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="D53" s="4" t="inlineStr">
-        <is>
-          <t>Industrial</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="n"/>
-      <c r="F53" s="6" t="n"/>
-      <c r="G53" s="5" t="n"/>
-      <c r="H53" s="4" t="n"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licota trolley 272,440 and more toolsmart.pk Licota listings (DOE 36x41/41x46, snap ring set, offset ring singles)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4c5Y1XBRj63SkdBZ73bUS
</commit_message>
<xml_diff>
--- a/quotes/PR-217-228/RFQ_PR217_PR228.xlsx
+++ b/quotes/PR-217-228/RFQ_PR217_PR228.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -538,19 +538,19 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>7 DRAWER TOOL TROLLEY</t>
+          <t>DOUBLE OPEN RING OFFSET WRENCH SET (12PCS)</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Licota (AWX series, empty)</t>
+          <t>Licota</t>
         </is>
       </c>
       <c r="E5" s="5" t="n"/>
@@ -560,11 +560,11 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>DOUBLE OPEN RING OFFSET WRENCH SET (12PCS)</t>
+          <t>DOUBLE OPEN END WRENCH 6 TO 32 (12 PCS SET)</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
@@ -582,11 +582,11 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>DOUBLE OPEN END WRENCH 6 TO 32 (12 PCS SET)</t>
+          <t>COMBINATION WRENCH 8 TO 32 (14 PCS SET)</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
@@ -604,15 +604,15 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>DOUBLE OPEN END WRENCH 36X41</t>
+          <t>HOLLOW PUNCH (3MM-25MM) (15PCS SET)</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
@@ -626,15 +626,15 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>DOUBLE OPEN END WRENCH 41X46</t>
+          <t>SHORT TYPE HEX KEY WRENCH SET (09PCS)</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
@@ -648,15 +648,15 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>COMBINATION WRENCH 8 TO 32 (14 PCS SET)</t>
+          <t>ALLEN HEX KEY 12MM</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
@@ -670,15 +670,15 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>HOLLOW PUNCH (3MM-25MM) (15PCS SET)</t>
+          <t>ALLEN (HEX) KEY 14MM</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
@@ -692,15 +692,15 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>SHORT TYPE HEX KEY WRENCH SET (09PCS)</t>
+          <t>ALLEN (HEX) KEY 16MM</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
@@ -714,15 +714,15 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>ALLEN HEX KEY 12MM</t>
+          <t>CIRCLIP PLIER INTERNAL STRAIGHT 230MM</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
@@ -736,11 +736,11 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>ALLEN (HEX) KEY 14MM</t>
+          <t>CIRCLIP PLIER EXTERNAL STRAIGHT 230MM</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
@@ -758,11 +758,11 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>ALLEN (HEX) KEY 16MM</t>
+          <t>PIPE WRENCH SIZE 10"</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
@@ -780,15 +780,15 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>CIRCLIP PLIER INTERNAL STRAIGHT 230MM</t>
+          <t>PIPE WRENCH SIZE 12"</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
@@ -802,15 +802,15 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>CIRCLIP PLIER EXTERNAL STRAIGHT 230MM</t>
+          <t>PIPE WRENCH SIZE 24"</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
@@ -824,15 +824,15 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>PIPE WRENCH SIZE 10"</t>
+          <t>PIPE WRENCH SIZE 36"</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
@@ -846,11 +846,11 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>PIPE WRENCH SIZE 12"</t>
+          <t>SLEDGE HAMMER 1 LBS WITH FIBREGLASS HANDLE</t>
         </is>
       </c>
       <c r="C19" s="4" t="n">
@@ -868,15 +868,15 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>PIPE WRENCH SIZE 24"</t>
+          <t>SLEDGE HAMMER 3 LBS WITH FIBREGLASS HANDLE</t>
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
@@ -890,15 +890,15 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>PIPE WRENCH SIZE 36"</t>
+          <t>SOFT FACE DEAD BLOW HAMMER 50MM</t>
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
@@ -912,11 +912,11 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>SLEDGE HAMMER 1 LBS WITH FIBREGLASS HANDLE</t>
+          <t>VICE GRIP PLIER 08"</t>
         </is>
       </c>
       <c r="C22" s="4" t="n">
@@ -934,15 +934,15 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>SLEDGE HAMMER 3 LBS WITH FIBREGLASS HANDLE</t>
+          <t>HEX IMPACT ADAPTOR 1/2" FEMALE TO 1/4" FEMALE</t>
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
@@ -956,11 +956,11 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>SOFT FACE DEAD BLOW HAMMER 50MM</t>
+          <t>UNIVERSAL PULLER 2-ARMED WITH HOOK BRAKE 21</t>
         </is>
       </c>
       <c r="C24" s="4" t="n">
@@ -978,15 +978,15 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>VICE GRIP PLIER 08"</t>
+          <t>UNIVERSAL PULLER 2-ARMED WITH HOOK BRAK 250</t>
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
@@ -1000,15 +1000,15 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>HEX IMPACT ADAPTOR 1/2" FEMALE TO 1/4" FEMALE</t>
+          <t>UNIVERSAL PULLER 2-ARMED 160 X 300 MM 5T</t>
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
@@ -1022,15 +1022,15 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>UNIVERSAL PULLER 2-ARMED WITH HOOK BRAKE 21</t>
+          <t>UNIVERSAL PULLER 2-ARMED 250 X 300 MM 7.5T</t>
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
@@ -1044,15 +1044,15 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>UNIVERSAL PULLER 2-ARMED WITH HOOK BRAK 250</t>
+          <t>INTERNAL EXTRACTOR WITH REINFORCED COLLAR</t>
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
@@ -1066,15 +1066,15 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>UNIVERSAL PULLER 2-ARMED 160 X 300 MM 5T</t>
+          <t>MECHANICAL PULLER 3 ARMED 200X200</t>
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
@@ -1088,11 +1088,11 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>UNIVERSAL PULLER 2-ARMED 250 X 300 MM 7.5T</t>
+          <t>MECHANICAL PULLER 3 ARMED 250X250</t>
         </is>
       </c>
       <c r="C30" s="4" t="n">
@@ -1110,11 +1110,11 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>INTERNAL EXTRACTOR WITH REINFORCED COLLAR</t>
+          <t>AIR GREASE GUN 500CC</t>
         </is>
       </c>
       <c r="C31" s="4" t="n">
@@ -1132,15 +1132,15 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>MECHANICAL PULLER 3 ARMED 200X200</t>
+          <t>GREASE PIPE 1/4"X12"</t>
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
@@ -1154,15 +1154,15 @@
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>MECHANICAL PULLER 3 ARMED 250X250</t>
+          <t>DOUBLE HANDLE GREASE NOZZLE</t>
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
@@ -1176,15 +1176,15 @@
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>AIR GREASE GUN 500CC</t>
+          <t>ALIGNING PRY BAR DIA 5/8" X 18" LENGTH</t>
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
@@ -1198,15 +1198,15 @@
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>GREASE PIPE 1/4"X12"</t>
+          <t>ADJUSTABLE WRENCH 15"</t>
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
@@ -1220,11 +1220,11 @@
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
-        <v>59</v>
+        <v>148</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>DOUBLE HANDLE GREASE NOZZLE</t>
+          <t>FLATE METAL SCRAPPER 50MM</t>
         </is>
       </c>
       <c r="C36" s="4" t="n">
@@ -1239,72 +1239,6 @@
       <c r="F36" s="6" t="n"/>
       <c r="G36" s="5" t="n"/>
       <c r="H36" s="4" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="n">
-        <v>62</v>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>ALIGNING PRY BAR DIA 5/8" X 18" LENGTH</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>Licota</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="n"/>
-      <c r="F37" s="6" t="n"/>
-      <c r="G37" s="5" t="n"/>
-      <c r="H37" s="4" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="n">
-        <v>63</v>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>ADJUSTABLE WRENCH 15"</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>Licota</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="n"/>
-      <c r="F38" s="6" t="n"/>
-      <c r="G38" s="5" t="n"/>
-      <c r="H38" s="4" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="n">
-        <v>148</v>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>FLATE METAL SCRAPPER 50MM</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>Licota</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="n"/>
-      <c r="F39" s="6" t="n"/>
-      <c r="G39" s="5" t="n"/>
-      <c r="H39" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
More toolsmart.pk Licota listings (short hex set, locking plier, pin punch)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4c5Y1XBRj63SkdBZ73bUS
</commit_message>
<xml_diff>
--- a/quotes/PR-217-228/RFQ_PR217_PR228.xlsx
+++ b/quotes/PR-217-228/RFQ_PR217_PR228.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -626,15 +626,15 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>SHORT TYPE HEX KEY WRENCH SET (09PCS)</t>
+          <t>ALLEN HEX KEY 12MM</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
@@ -648,11 +648,11 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>ALLEN HEX KEY 12MM</t>
+          <t>ALLEN (HEX) KEY 14MM</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
@@ -670,11 +670,11 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>ALLEN (HEX) KEY 14MM</t>
+          <t>ALLEN (HEX) KEY 16MM</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
@@ -692,15 +692,15 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>ALLEN (HEX) KEY 16MM</t>
+          <t>CIRCLIP PLIER INTERNAL STRAIGHT 230MM</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
@@ -714,15 +714,15 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>CIRCLIP PLIER INTERNAL STRAIGHT 230MM</t>
+          <t>CIRCLIP PLIER EXTERNAL STRAIGHT 230MM</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
@@ -736,11 +736,11 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>CIRCLIP PLIER EXTERNAL STRAIGHT 230MM</t>
+          <t>PIPE WRENCH SIZE 10"</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
@@ -758,11 +758,11 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>PIPE WRENCH SIZE 10"</t>
+          <t>PIPE WRENCH SIZE 12"</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
@@ -780,15 +780,15 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>PIPE WRENCH SIZE 12"</t>
+          <t>PIPE WRENCH SIZE 24"</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
@@ -802,11 +802,11 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>PIPE WRENCH SIZE 24"</t>
+          <t>PIPE WRENCH SIZE 36"</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
@@ -824,15 +824,15 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>PIPE WRENCH SIZE 36"</t>
+          <t>SLEDGE HAMMER 1 LBS WITH FIBREGLASS HANDLE</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
@@ -846,11 +846,11 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>SLEDGE HAMMER 1 LBS WITH FIBREGLASS HANDLE</t>
+          <t>SLEDGE HAMMER 3 LBS WITH FIBREGLASS HANDLE</t>
         </is>
       </c>
       <c r="C19" s="4" t="n">
@@ -868,11 +868,11 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>SLEDGE HAMMER 3 LBS WITH FIBREGLASS HANDLE</t>
+          <t>SOFT FACE DEAD BLOW HAMMER 50MM</t>
         </is>
       </c>
       <c r="C20" s="4" t="n">
@@ -890,11 +890,11 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>SOFT FACE DEAD BLOW HAMMER 50MM</t>
+          <t>VICE GRIP PLIER 08"</t>
         </is>
       </c>
       <c r="C21" s="4" t="n">
@@ -912,15 +912,15 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>VICE GRIP PLIER 08"</t>
+          <t>HEX IMPACT ADAPTOR 1/2" FEMALE TO 1/4" FEMALE</t>
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
@@ -934,15 +934,15 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>HEX IMPACT ADAPTOR 1/2" FEMALE TO 1/4" FEMALE</t>
+          <t>UNIVERSAL PULLER 2-ARMED WITH HOOK BRAKE 21</t>
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
@@ -956,15 +956,15 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>UNIVERSAL PULLER 2-ARMED WITH HOOK BRAKE 21</t>
+          <t>UNIVERSAL PULLER 2-ARMED WITH HOOK BRAK 250</t>
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
@@ -978,15 +978,15 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>UNIVERSAL PULLER 2-ARMED WITH HOOK BRAK 250</t>
+          <t>UNIVERSAL PULLER 2-ARMED 160 X 300 MM 5T</t>
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
@@ -1000,11 +1000,11 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>UNIVERSAL PULLER 2-ARMED 160 X 300 MM 5T</t>
+          <t>UNIVERSAL PULLER 2-ARMED 250 X 300 MM 7.5T</t>
         </is>
       </c>
       <c r="C26" s="4" t="n">
@@ -1022,11 +1022,11 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>UNIVERSAL PULLER 2-ARMED 250 X 300 MM 7.5T</t>
+          <t>INTERNAL EXTRACTOR WITH REINFORCED COLLAR</t>
         </is>
       </c>
       <c r="C27" s="4" t="n">
@@ -1044,15 +1044,15 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>INTERNAL EXTRACTOR WITH REINFORCED COLLAR</t>
+          <t>MECHANICAL PULLER 3 ARMED 200X200</t>
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
@@ -1066,15 +1066,15 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>MECHANICAL PULLER 3 ARMED 200X200</t>
+          <t>MECHANICAL PULLER 3 ARMED 250X250</t>
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
@@ -1088,11 +1088,11 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>MECHANICAL PULLER 3 ARMED 250X250</t>
+          <t>AIR GREASE GUN 500CC</t>
         </is>
       </c>
       <c r="C30" s="4" t="n">
@@ -1110,15 +1110,15 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>AIR GREASE GUN 500CC</t>
+          <t>GREASE PIPE 1/4"X12"</t>
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
@@ -1132,11 +1132,11 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>GREASE PIPE 1/4"X12"</t>
+          <t>DOUBLE HANDLE GREASE NOZZLE</t>
         </is>
       </c>
       <c r="C32" s="4" t="n">
@@ -1154,15 +1154,15 @@
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>DOUBLE HANDLE GREASE NOZZLE</t>
+          <t>ALIGNING PRY BAR DIA 5/8" X 18" LENGTH</t>
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
@@ -1176,15 +1176,15 @@
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>ALIGNING PRY BAR DIA 5/8" X 18" LENGTH</t>
+          <t>ADJUSTABLE WRENCH 15"</t>
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
@@ -1198,15 +1198,15 @@
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>63</v>
+        <v>148</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>ADJUSTABLE WRENCH 15"</t>
+          <t>FLATE METAL SCRAPPER 50MM</t>
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
@@ -1217,28 +1217,6 @@
       <c r="F35" s="6" t="n"/>
       <c r="G35" s="5" t="n"/>
       <c r="H35" s="4" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="n">
-        <v>148</v>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>FLATE METAL SCRAPPER 50MM</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>Licota</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="n"/>
-      <c r="F36" s="6" t="n"/>
-      <c r="G36" s="5" t="n"/>
-      <c r="H36" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Verify remaining items from UAE/UK/US listings (AED x90 basis), Taiwan where brand unclear
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4c5Y1XBRj63SkdBZ73bUS
</commit_message>
<xml_diff>
--- a/quotes/PR-217-228/RFQ_PR217_PR228.xlsx
+++ b/quotes/PR-217-228/RFQ_PR217_PR228.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -560,11 +560,11 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>ALLEN HEX KEY 12MM</t>
+          <t>ALLEN (HEX) KEY 14MM</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
@@ -582,11 +582,11 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>ALLEN (HEX) KEY 14MM</t>
+          <t>ALLEN (HEX) KEY 16MM</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
@@ -604,15 +604,15 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>ALLEN (HEX) KEY 16MM</t>
+          <t>CIRCLIP PLIER INTERNAL STRAIGHT 230MM</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
@@ -626,15 +626,15 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>CIRCLIP PLIER INTERNAL STRAIGHT 230MM</t>
+          <t>CIRCLIP PLIER EXTERNAL STRAIGHT 230MM</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
@@ -648,11 +648,11 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>CIRCLIP PLIER EXTERNAL STRAIGHT 230MM</t>
+          <t>VICE GRIP PLIER 08"</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
@@ -670,15 +670,15 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>VICE GRIP PLIER 08"</t>
+          <t>HEX IMPACT ADAPTOR 1/2" FEMALE TO 1/4" FEMALE</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
@@ -692,15 +692,15 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>HEX IMPACT ADAPTOR 1/2" FEMALE TO 1/4" FEMALE</t>
+          <t>INTERNAL EXTRACTOR WITH REINFORCED COLLAR</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
@@ -714,15 +714,15 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>UNIVERSAL PULLER 2-ARMED WITH HOOK BRAKE 21</t>
+          <t>AIR GREASE GUN 500CC</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
@@ -736,15 +736,15 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>UNIVERSAL PULLER 2-ARMED WITH HOOK BRAK 250</t>
+          <t>GREASE PIPE 1/4"X12"</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
@@ -758,15 +758,15 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>UNIVERSAL PULLER 2-ARMED 160 X 300 MM 5T</t>
+          <t>DOUBLE HANDLE GREASE NOZZLE</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
@@ -777,116 +777,6 @@
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="5" t="n"/>
       <c r="H15" s="4" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>UNIVERSAL PULLER 2-ARMED 250 X 300 MM 7.5T</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Licota</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="6" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="4" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="n">
-        <v>51</v>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>INTERNAL EXTRACTOR WITH REINFORCED COLLAR</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Licota</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="6" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="4" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="n">
-        <v>56</v>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>AIR GREASE GUN 500CC</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Licota</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="6" t="n"/>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="4" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="n">
-        <v>58</v>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>GREASE PIPE 1/4"X12"</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Licota</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="6" t="n"/>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="4" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="n">
-        <v>59</v>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>DOUBLE HANDLE GREASE NOZZLE</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Licota</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="5" t="n"/>
-      <c r="H20" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -899,7 +789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -970,19 +860,19 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>4</v>
+        <v>74</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>DRILL BIT 08 MM (Yato or any Good brand taiwan)</t>
+          <t>HSS DRILL BITS 1/16-1/2" 29 PCS SET</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Dormer A002</t>
+          <t>Dormer A095 (A002 x29)</t>
         </is>
       </c>
       <c r="E5" s="5" t="n"/>
@@ -992,11 +882,11 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BITS 1/16-1/2" 29 PCS SET</t>
+          <t>HSS DRILL BIT 15.5MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
@@ -1004,7 +894,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Dormer A095 (A002 x29)</t>
+          <t>Dormer A130</t>
         </is>
       </c>
       <c r="E6" s="5" t="n"/>
@@ -1014,11 +904,11 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 14MM TAPER SHANK</t>
+          <t>HSS DRILL BIT 16.5MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
@@ -1036,15 +926,15 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 15MM TAPER SHANK</t>
+          <t>HSS DRILL BIT 21MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
@@ -1058,15 +948,15 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 15.5MM TAPER SHANK</t>
+          <t>HSS DRILL BIT 30MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
@@ -1080,15 +970,15 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 16MM TAPER SHANK</t>
+          <t>HSS DRILL BIT 35MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
@@ -1102,19 +992,19 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 16.5MM TAPER SHANK</t>
+          <t>TAP SET 1/2" BSPF LEFT HAND (Dormer)</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Dormer A130</t>
+          <t>Dormer</t>
         </is>
       </c>
       <c r="E11" s="5" t="n"/>
@@ -1124,19 +1014,19 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 17MM TAPER SHANK</t>
+          <t>TAP SET 1/2" BSPF RIGHT HAND</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Dormer A130</t>
+          <t>Dormer</t>
         </is>
       </c>
       <c r="E12" s="5" t="n"/>
@@ -1146,19 +1036,19 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>81</v>
+        <v>100</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 17.5MM TAPER SHANK</t>
+          <t>TAP SET 3/8" BSPF</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Dormer A130</t>
+          <t>Dormer</t>
         </is>
       </c>
       <c r="E13" s="5" t="n"/>
@@ -1168,19 +1058,19 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>82</v>
+        <v>179</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 19MM TAPER SHANK</t>
+          <t>TAP SET 1" BSPF LEFT HAND</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Dormer A130</t>
+          <t>Dormer</t>
         </is>
       </c>
       <c r="E14" s="5" t="n"/>
@@ -1190,11 +1080,11 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>83</v>
+        <v>180</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 21MM TAPER SHANK</t>
+          <t>TAP SET 1" BSPF RIGHT HAND</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
@@ -1202,7 +1092,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Dormer A130</t>
+          <t>Dormer</t>
         </is>
       </c>
       <c r="E15" s="5" t="n"/>
@@ -1212,11 +1102,11 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>84</v>
+        <v>181</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 25MM TAPER SHANK</t>
+          <t>TAP SET 1-1/4" BSPF LEFT HAND</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
@@ -1224,7 +1114,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Dormer A130</t>
+          <t>Dormer</t>
         </is>
       </c>
       <c r="E16" s="5" t="n"/>
@@ -1234,11 +1124,11 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>85</v>
+        <v>182</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 30MM TAPER SHANK</t>
+          <t>TAP SET 1-1/4" BSPF RIGHT HAND</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
@@ -1246,7 +1136,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Dormer A130</t>
+          <t>Dormer</t>
         </is>
       </c>
       <c r="E17" s="5" t="n"/>
@@ -1256,11 +1146,11 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>86</v>
+        <v>188</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 32MM TAPER SHANK</t>
+          <t>TAP SET M18</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
@@ -1268,7 +1158,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Dormer A130</t>
+          <t>Dormer</t>
         </is>
       </c>
       <c r="E18" s="5" t="n"/>
@@ -1278,19 +1168,19 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>87</v>
+        <v>210</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 35MM TAPER SHANK</t>
+          <t>END MILL CUTTER SIZE 18MM</t>
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Dormer A130</t>
+          <t>Dormer</t>
         </is>
       </c>
       <c r="E19" s="5" t="n"/>
@@ -1300,11 +1190,11 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>98</v>
+        <v>211</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>TAP SET 1/2" BSPF LEFT HAND (Dormer)</t>
+          <t>END MILL CUTTER SIZE 22MM</t>
         </is>
       </c>
       <c r="C20" s="4" t="n">
@@ -1322,15 +1212,15 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>99</v>
+        <v>228</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>TAP SET 1/2" BSPF RIGHT HAND</t>
+          <t>HSS TOOL 16MMX16MMX200MM</t>
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
@@ -1341,468 +1231,6 @@
       <c r="F21" s="6" t="n"/>
       <c r="G21" s="5" t="n"/>
       <c r="H21" s="4" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>TAP SET 3/8" BSPF</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Dormer</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="n"/>
-      <c r="F22" s="6" t="n"/>
-      <c r="G22" s="5" t="n"/>
-      <c r="H22" s="4" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="n">
-        <v>101</v>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>TAP SET 1/4" BSPF</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>Dormer</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="6" t="n"/>
-      <c r="G23" s="5" t="n"/>
-      <c r="H23" s="4" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="n">
-        <v>102</v>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>TAP SET 1/8" BSPF</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>Dormer</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="n"/>
-      <c r="F24" s="6" t="n"/>
-      <c r="G24" s="5" t="n"/>
-      <c r="H24" s="4" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="n">
-        <v>179</v>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>TAP SET 1" BSPF LEFT HAND</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>Dormer</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="n"/>
-      <c r="F25" s="6" t="n"/>
-      <c r="G25" s="5" t="n"/>
-      <c r="H25" s="4" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="n">
-        <v>180</v>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>TAP SET 1" BSPF RIGHT HAND</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>Dormer</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="n"/>
-      <c r="F26" s="6" t="n"/>
-      <c r="G26" s="5" t="n"/>
-      <c r="H26" s="4" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="n">
-        <v>181</v>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>TAP SET 1-1/4" BSPF LEFT HAND</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>Dormer</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="n"/>
-      <c r="F27" s="6" t="n"/>
-      <c r="G27" s="5" t="n"/>
-      <c r="H27" s="4" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="n">
-        <v>182</v>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>TAP SET 1-1/4" BSPF RIGHT HAND</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>Dormer</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="n"/>
-      <c r="F28" s="6" t="n"/>
-      <c r="G28" s="5" t="n"/>
-      <c r="H28" s="4" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="n">
-        <v>204</v>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>END MILL CUTTER SIZE 5MM</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>Dormer C-series HSS-Co</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="n"/>
-      <c r="F29" s="6" t="n"/>
-      <c r="G29" s="5" t="n"/>
-      <c r="H29" s="4" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="n">
-        <v>205</v>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>END MILL CUTTER SIZE 6MM</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>Dormer C-series HSS-Co</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="n"/>
-      <c r="F30" s="6" t="n"/>
-      <c r="G30" s="5" t="n"/>
-      <c r="H30" s="4" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="n">
-        <v>206</v>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>END MILL CUTTER SIZE 8MM</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>Dormer C-series HSS-Co</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="n"/>
-      <c r="F31" s="6" t="n"/>
-      <c r="G31" s="5" t="n"/>
-      <c r="H31" s="4" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="n">
-        <v>207</v>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>END MILL CUTTER SIZE 10MM</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>Dormer C-series HSS-Co</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="n"/>
-      <c r="F32" s="6" t="n"/>
-      <c r="G32" s="5" t="n"/>
-      <c r="H32" s="4" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="n">
-        <v>209</v>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>END MILL CUTTER SIZE 16MM</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>Dormer C-series HSS-Co</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="n"/>
-      <c r="F33" s="6" t="n"/>
-      <c r="G33" s="5" t="n"/>
-      <c r="H33" s="4" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="n">
-        <v>210</v>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>END MILL CUTTER SIZE 18MM</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>Dormer C-series HSS-Co</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="n"/>
-      <c r="F34" s="6" t="n"/>
-      <c r="G34" s="5" t="n"/>
-      <c r="H34" s="4" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="n">
-        <v>211</v>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>END MILL CUTTER SIZE 22MM</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>Dormer C-series HSS-Co</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="n"/>
-      <c r="F35" s="6" t="n"/>
-      <c r="G35" s="5" t="n"/>
-      <c r="H35" s="4" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="n">
-        <v>212</v>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>END MILL CUTTER SIZE 25MM</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>Dormer C-series HSS-Co</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="n"/>
-      <c r="F36" s="6" t="n"/>
-      <c r="G36" s="5" t="n"/>
-      <c r="H36" s="4" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="n">
-        <v>225</v>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>HSS TOOL 08X08X200MM</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>Dormer</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="n"/>
-      <c r="F37" s="6" t="n"/>
-      <c r="G37" s="5" t="n"/>
-      <c r="H37" s="4" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="n">
-        <v>226</v>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>HSS TOOL 10MMX10MMX200MM</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>Dormer</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="n"/>
-      <c r="F38" s="6" t="n"/>
-      <c r="G38" s="5" t="n"/>
-      <c r="H38" s="4" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="n">
-        <v>227</v>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>HSS TOOL 12MMX12MMX200MM</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>Dormer</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="n"/>
-      <c r="F39" s="6" t="n"/>
-      <c r="G39" s="5" t="n"/>
-      <c r="H39" s="4" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="n">
-        <v>228</v>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>HSS TOOL 16MMX16MMX200MM</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>Dormer</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="n"/>
-      <c r="F40" s="6" t="n"/>
-      <c r="G40" s="5" t="n"/>
-      <c r="H40" s="4" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="n">
-        <v>229</v>
-      </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>HSS PARTING OFF TOOL 1/8" X 3/4" X 8"</t>
-        </is>
-      </c>
-      <c r="C41" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>Dormer</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="n"/>
-      <c r="F41" s="6" t="n"/>
-      <c r="G41" s="5" t="n"/>
-      <c r="H41" s="4" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="n">
-        <v>240</v>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>DRILL BIT 4MM</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>Dormer A002</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="n"/>
-      <c r="F42" s="6" t="n"/>
-      <c r="G42" s="5" t="n"/>
-      <c r="H42" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1815,7 +1243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1886,19 +1314,19 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>2</v>
+        <v>45</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>STEEL NAIL 1-1/2" Taiwan</t>
+          <t>ROUNDE FILE 12"</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Generic (Taiwan)</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E5" s="5" t="n"/>
@@ -1908,19 +1336,19 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>UNIVERSAL PULLER 2-ARMED WITH HOOK BRAKE 21</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>MECHANICAL JACK 5 TON (Japan or Germany)</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Masada (Japan)</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E6" s="5" t="n"/>
@@ -1930,19 +1358,19 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>MECHANICAL JACK 03 TONS (Japan or germany)</t>
+          <t>UNIVERSAL PULLER 2-ARMED 160 X 300 MM 5T</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Masada (Japan)</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E7" s="5" t="n"/>
@@ -1952,19 +1380,19 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>CORDLESS IMPACT WRENCH 350N (Bosch)</t>
+          <t>UNIVERSAL PULLER 2-ARMED 250 X 300 MM 7.5T</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Bosch Professional GDS 18V-350</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E8" s="5" t="n"/>
@@ -1974,15 +1402,15 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>ROUNDE FILE 12"</t>
+          <t>MANUAL GREASE GUN 5KG</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
@@ -1996,11 +1424,11 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>MANUAL GREASE GUN 5KG</t>
+          <t>REVOLVING CENTRE MT4</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
@@ -2008,7 +1436,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E10" s="5" t="n"/>
@@ -2018,11 +1446,11 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>66</v>
+        <v>88</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>REVOLVING CENTRE MT4</t>
+          <t>MORSE TAPER EXTENSION SOCKET SLEEVE ADAPT</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
@@ -2030,7 +1458,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Vertex (Taiwan)</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E11" s="5" t="n"/>
@@ -2040,11 +1468,11 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>67</v>
+        <v>89</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>REVOLVING CENTRE MT3</t>
+          <t>MORSE TAPER EXTENSION SOCKET SLEEVE ADAPT</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
@@ -2052,7 +1480,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Vertex (Taiwan)</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E12" s="5" t="n"/>
@@ -2062,11 +1490,11 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>CIRCUMFERENCE TAPE (60-950) (D20-300)</t>
+          <t>MORSE TAPER EXTENSION SOCKET SLEEVE ADAPT</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
@@ -2074,7 +1502,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Insize</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E13" s="5" t="n"/>
@@ -2084,19 +1512,19 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>70</v>
+        <v>91</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>CIRCUMFERENCE TAPE (940-2200) (D300-700)</t>
+          <t>DEAD CENTRE DIAMOND TIP M2</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Insize</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E14" s="5" t="n"/>
@@ -2106,11 +1534,11 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>MORSE TAPER EXTENSION SOCKET SLEEVE ADAPT</t>
+          <t>VERNIER DEPTH GUAGE 250MM GRADUATION 0.02M</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
@@ -2118,7 +1546,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Vertex (Taiwan)</t>
+          <t>Insize</t>
         </is>
       </c>
       <c r="E15" s="5" t="n"/>
@@ -2128,11 +1556,11 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>MORSE TAPER EXTENSION SOCKET SLEEVE ADAPT</t>
+          <t>CORDLESS DRILL DRIVER 150NM Bosch</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
@@ -2140,7 +1568,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Vertex (Taiwan)</t>
+          <t>Bosch Professional</t>
         </is>
       </c>
       <c r="E16" s="5" t="n"/>
@@ -2150,19 +1578,19 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>MORSE TAPER EXTENSION SOCKET SLEEVE ADAPT</t>
+          <t>C-CLAMP 12"</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Vertex (Taiwan)</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E17" s="5" t="n"/>
@@ -2172,19 +1600,19 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>91</v>
+        <v>109</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>DEAD CENTRE DIAMOND TIP M2</t>
+          <t>MAGNET SPIRIT LEVEL 12"</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Vertex (Taiwan)</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E18" s="5" t="n"/>
@@ -2194,11 +1622,11 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>92</v>
+        <v>123</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>DEAD CENTRE DIAMOND TIP M3</t>
+          <t>TIG WELDING TORCH AIR-COOLED 5METER</t>
         </is>
       </c>
       <c r="C19" s="4" t="n">
@@ -2206,7 +1634,7 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Vertex (Taiwan)</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E19" s="5" t="n"/>
@@ -2216,19 +1644,19 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>96</v>
+        <v>128</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>VERNIER DEPTH GUAGE 250MM GRADUATION 0.02M</t>
+          <t>CERAMIC CUP NO.6</t>
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Insize</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E20" s="5" t="n"/>
@@ -2238,19 +1666,19 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>97</v>
+        <v>129</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>CORDLESS DRILL DRIVER 150NM Bosch</t>
+          <t>CERAMIC CUP NO.7</t>
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Bosch Professional</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E21" s="5" t="n"/>
@@ -2260,19 +1688,19 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>107</v>
+        <v>142</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>C-CLAMP 12"</t>
+          <t>GRINDER WHEEL ALUMINIUM OXIDE GRIT 24</t>
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E22" s="5" t="n"/>
@@ -2282,19 +1710,19 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>109</v>
+        <v>143</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>MAGNET SPIRIT LEVEL 12"</t>
+          <t>GRINDER WHEEL ALUMINIUM OXIDE GRIT 60</t>
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E23" s="5" t="n"/>
@@ -2304,11 +1732,11 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>183</v>
+        <v>144</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>TAP SET M6</t>
+          <t>GRINDER WHEEL SILICON CARBIDE</t>
         </is>
       </c>
       <c r="C24" s="4" t="n">
@@ -2316,7 +1744,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E24" s="5" t="n"/>
@@ -2326,19 +1754,19 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>184</v>
+        <v>161</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>TAP SET M8</t>
+          <t>ANCHOR BOLT 12X120</t>
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>3</v>
+        <v>150</v>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E25" s="5" t="n"/>
@@ -2348,19 +1776,19 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>185</v>
+        <v>162</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>TAP SET M10</t>
+          <t>ANCHOR BOLT 12X160</t>
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>3</v>
+        <v>150</v>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E26" s="5" t="n"/>
@@ -2370,11 +1798,11 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>TAP SET M12</t>
+          <t>TAP SET M8</t>
         </is>
       </c>
       <c r="C27" s="4" t="n">
@@ -2392,11 +1820,11 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>TAP SET M16</t>
+          <t>INSIDE CALIPER 20"</t>
         </is>
       </c>
       <c r="C28" s="4" t="n">
@@ -2404,7 +1832,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Insize</t>
         </is>
       </c>
       <c r="E28" s="5" t="n"/>
@@ -2414,19 +1842,19 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>TAP SET M18</t>
+          <t>OUTSIDE CALIPER 20"</t>
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Insize</t>
         </is>
       </c>
       <c r="E29" s="5" t="n"/>
@@ -2436,15 +1864,15 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>189</v>
+        <v>213</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>TAP SET M20</t>
+          <t>DIE NUT SIZE 5MM</t>
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
@@ -2458,11 +1886,11 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>190</v>
+        <v>214</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>TAP HANDLE</t>
+          <t>DIE NUT SIZE 6MM</t>
         </is>
       </c>
       <c r="C31" s="4" t="n">
@@ -2480,11 +1908,11 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>191</v>
+        <v>215</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>TAP HANDLE</t>
+          <t>DIE NUT SIZE 8MM</t>
         </is>
       </c>
       <c r="C32" s="4" t="n">
@@ -2502,19 +1930,19 @@
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>192</v>
+        <v>216</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>INSIDE CALIPER 06"</t>
+          <t>DIE NUT SIZE 10MM</t>
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Generic (Taiwan)</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E33" s="5" t="n"/>
@@ -2524,11 +1952,11 @@
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>193</v>
+        <v>217</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>INSIDE CALIPER 20"</t>
+          <t>DIE NUT SIZE 12MM</t>
         </is>
       </c>
       <c r="C34" s="4" t="n">
@@ -2536,7 +1964,7 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Generic (Taiwan)</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E34" s="5" t="n"/>
@@ -2546,19 +1974,19 @@
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>194</v>
+        <v>219</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>OUTSIDE CALIPER 06"</t>
+          <t>DIE NUT HANDLE SMALL</t>
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Generic (Taiwan)</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E35" s="5" t="n"/>
@@ -2568,19 +1996,19 @@
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
-        <v>195</v>
+        <v>220</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>OUTSIDE CALIPER 20"</t>
+          <t>DIE NUT HANDLE MEDIUM</t>
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Generic (Taiwan)</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E36" s="5" t="n"/>
@@ -2590,15 +2018,15 @@
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
-        <v>196</v>
+        <v>221</v>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>RACHET TAP HANDLE</t>
+          <t>DIE NUT HANDLE LARGE</t>
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
@@ -2612,11 +2040,11 @@
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
-        <v>213</v>
+        <v>224</v>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>DIE NUT SIZE 5MM</t>
+          <t>BENCH VISE 12"</t>
         </is>
       </c>
       <c r="C38" s="4" t="n">
@@ -2624,7 +2052,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E38" s="5" t="n"/>
@@ -2634,19 +2062,19 @@
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>DIE NUT SIZE 6MM</t>
+          <t>HSS TOOL 10MMX10MMX200MM</t>
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E39" s="5" t="n"/>
@@ -2656,19 +2084,19 @@
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>DIE NUT SIZE 8MM</t>
+          <t>HSS TOOL 12MMX12MMX200MM</t>
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E40" s="5" t="n"/>
@@ -2678,179 +2106,25 @@
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
-        <v>216</v>
+        <v>229</v>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>DIE NUT SIZE 10MM</t>
+          <t>HSS PARTING OFF TOOL 1/8" X 3/4" X 8"</t>
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E41" s="5" t="n"/>
       <c r="F41" s="6" t="n"/>
       <c r="G41" s="5" t="n"/>
       <c r="H41" s="4" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="n">
-        <v>217</v>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>DIE NUT SIZE 12MM</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="n"/>
-      <c r="F42" s="6" t="n"/>
-      <c r="G42" s="5" t="n"/>
-      <c r="H42" s="4" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="n">
-        <v>218</v>
-      </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>DIE NUT SIZE 16MM</t>
-        </is>
-      </c>
-      <c r="C43" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="n"/>
-      <c r="F43" s="6" t="n"/>
-      <c r="G43" s="5" t="n"/>
-      <c r="H43" s="4" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="n">
-        <v>219</v>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>DIE NUT HANDLE SMALL</t>
-        </is>
-      </c>
-      <c r="C44" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="n"/>
-      <c r="F44" s="6" t="n"/>
-      <c r="G44" s="5" t="n"/>
-      <c r="H44" s="4" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="n">
-        <v>220</v>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>DIE NUT HANDLE MEDIUM</t>
-        </is>
-      </c>
-      <c r="C45" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="n"/>
-      <c r="F45" s="6" t="n"/>
-      <c r="G45" s="5" t="n"/>
-      <c r="H45" s="4" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="n">
-        <v>221</v>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>DIE NUT HANDLE LARGE</t>
-        </is>
-      </c>
-      <c r="C46" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>Yato</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="n"/>
-      <c r="F46" s="6" t="n"/>
-      <c r="G46" s="5" t="n"/>
-      <c r="H46" s="4" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="n">
-        <v>222</v>
-      </c>
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>3 JAW CHUCK 4"</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>Vertex (Taiwan)</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="n"/>
-      <c r="F47" s="6" t="n"/>
-      <c r="G47" s="5" t="n"/>
-      <c r="H47" s="4" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="n">
-        <v>224</v>
-      </c>
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>BENCH VISE 12"</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>Yato (heavy)</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="n"/>
-      <c r="F48" s="6" t="n"/>
-      <c r="G48" s="5" t="n"/>
-      <c r="H48" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2863,7 +2137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2956,19 +2230,19 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>HOLLOW PUNCH (3MM-25MM) (15PCS SET)</t>
+          <t>STEEL NAIL 1-1/2" Taiwan</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Harden</t>
+          <t>Generic</t>
         </is>
       </c>
       <c r="E6" s="5" t="n"/>
@@ -2978,19 +2252,19 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>SLEDGE HAMMER 1 LBS WITH FIBREGLASS HANDLE</t>
+          <t>HOLLOW PUNCH (3MM-25MM) (15PCS SET)</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Harden</t>
         </is>
       </c>
       <c r="E7" s="5" t="n"/>
@@ -3000,15 +2274,15 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>STEEL MEASURMENT TAPE 100M</t>
+          <t>SLEDGE HAMMER 1 LBS WITH FIBREGLASS HANDLE</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
@@ -3022,19 +2296,19 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>ALIGNING PRY BAR DIA 5/8" X 18" LENGTH</t>
+          <t>STEEL MEASURMENT TAPE 100M</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Ingco</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E9" s="5" t="n"/>
@@ -3044,15 +2318,15 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>HSS COBALT DRILL SET 1-13MM 25 PCS</t>
+          <t>ALIGNING PRY BAR DIA 5/8" X 18" LENGTH</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
@@ -3066,19 +2340,19 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>104</v>
+        <v>73</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>WELDING HELMET (FLIP FRONT)</t>
+          <t>HSS COBALT DRILL SET 1-13MM 25 PCS</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Ingco</t>
         </is>
       </c>
       <c r="E11" s="5" t="n"/>
@@ -3088,19 +2362,19 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>CARBON STEEL RIGHT ANGLE 150MM</t>
+          <t>WELDING HELMET (FLIP FRONT)</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Ingco</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="E12" s="5" t="n"/>
@@ -3132,15 +2406,15 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>FUEL GAS REGULATOR 0-2.5 BAR</t>
+          <t>OXYGEN HOSE 08MM ID</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
@@ -3154,11 +2428,11 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>OXYGEN HOSE 08MM ID</t>
+          <t>ACETYLENE GAS HOSE 08 ID</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
@@ -3176,15 +2450,15 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>ACETYLENE GAS HOSE 08 ID</t>
+          <t>CYLINDER KEY/SPANNER</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
@@ -3198,19 +2472,19 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER KEY/SPANNER</t>
+          <t>AC/DC SINGLE PHASE WELDING PLANT 300 AMP</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>WACTA20</t>
         </is>
       </c>
       <c r="E17" s="5" t="n"/>
@@ -3220,15 +2494,15 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>TIP CLEANER FOR GAS WELDING TORCH</t>
+          <t>TORCH HEAD ARGON WELDING</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
@@ -3242,19 +2516,19 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>AC/DC SINGLE PHASE WELDING PLANT 300 AMP</t>
+          <t>ARGON GAS HOSE 06MM</t>
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>WACTA20</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="E19" s="5" t="n"/>
@@ -3264,15 +2538,15 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>123</v>
+        <v>139</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>TIG WELDING TORCH AIR-COOLED 5METER</t>
+          <t>BUFFING DISC 125MM</t>
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
@@ -3286,19 +2560,19 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>TORCH HEAD ARGON WELDING</t>
+          <t>COTTON ROPE 2MM</t>
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>2</v>
+        <v>500</v>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Local</t>
         </is>
       </c>
       <c r="E21" s="5" t="n"/>
@@ -3308,11 +2582,11 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>125</v>
+        <v>154</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>COLLECT OF ARGON 2.4MM</t>
+          <t>RED OXIDE POWDER</t>
         </is>
       </c>
       <c r="C22" s="4" t="n">
@@ -3330,19 +2604,19 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>126</v>
+        <v>159</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>COLLECT BODY FOR ARGON 2.4MM</t>
+          <t>CUT PIECES OF CLOTHS FOR CLEANING</t>
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>12</v>
+        <v>100</v>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Local</t>
         </is>
       </c>
       <c r="E23" s="5" t="n"/>
@@ -3352,19 +2626,19 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>127</v>
+        <v>160</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>CERAMIC CUP NO.5</t>
+          <t>ANCHOR BOLT 10X110</t>
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>6</v>
+        <v>150</v>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>SMT</t>
         </is>
       </c>
       <c r="E24" s="5" t="n"/>
@@ -3374,19 +2648,19 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>128</v>
+        <v>164</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>CERAMIC CUP NO.6</t>
+          <t>WELDING RODS 2.5MM E6013, NO 10 Zodian</t>
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Zodian</t>
         </is>
       </c>
       <c r="E25" s="5" t="n"/>
@@ -3396,19 +2670,19 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>129</v>
+        <v>165</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>CERAMIC CUP NO.7</t>
+          <t>WELDING RODS 3.25MM E6013 NO 12</t>
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Zodian</t>
         </is>
       </c>
       <c r="E26" s="5" t="n"/>
@@ -3418,19 +2692,19 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>130</v>
+        <v>166</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>TUNGSTEN ELECTRODE 2.4MM</t>
+          <t>WELDING RODS 2.5MM E7018 NO-10</t>
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Fortrex</t>
         </is>
       </c>
       <c r="E27" s="5" t="n"/>
@@ -3440,19 +2714,19 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>132</v>
+        <v>167</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>ARGON GAS HOSE 06MM</t>
+          <t>SS WELDING RODS 309L-16 2.6MM NO.12</t>
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Stainarc</t>
         </is>
       </c>
       <c r="E28" s="5" t="n"/>
@@ -3462,19 +2736,19 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>133</v>
+        <v>168</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>GAS HOSE CONNECTOR</t>
+          <t>SS WELDING RODS 316L-16 2.6MM NO.12</t>
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Stainarc</t>
         </is>
       </c>
       <c r="E29" s="5" t="n"/>
@@ -3484,19 +2758,19 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>134</v>
+        <v>177</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>SHORT SLEEVE TIG WELDING GLOVES 10-INCH</t>
+          <t>BLIND RIVETS 04MMX25MM (1000PCS)</t>
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Generic</t>
         </is>
       </c>
       <c r="E30" s="5" t="n"/>
@@ -3506,19 +2780,19 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>139</v>
+        <v>202</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>BUFFING DISC 125MM</t>
+          <t>NEEDLE FILE (5PCS SET)</t>
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E31" s="5" t="n"/>
@@ -3528,19 +2802,19 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>140</v>
+        <v>230</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>BRASS PLATED CUP WIRE BRUSH 125MM</t>
+          <t>HYDRAULIC JACK 3 TON</t>
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Ronix</t>
         </is>
       </c>
       <c r="E32" s="5" t="n"/>
@@ -3550,11 +2824,11 @@
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>142</v>
+        <v>234</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>GRINDER WHEEL ALUMINIUM OXIDE GRIT 24</t>
+          <t>WELDING ELCTRODE HOLDER 1000 AMP</t>
         </is>
       </c>
       <c r="C33" s="4" t="n">
@@ -3562,7 +2836,7 @@
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Norton</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E33" s="5" t="n"/>
@@ -3572,11 +2846,11 @@
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>143</v>
+        <v>235</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>GRINDER WHEEL ALUMINIUM OXIDE GRIT 60</t>
+          <t>EARTH CLAMP 1000 AMP</t>
         </is>
       </c>
       <c r="C34" s="4" t="n">
@@ -3584,7 +2858,7 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Norton</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="E34" s="5" t="n"/>
@@ -3594,19 +2868,19 @@
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>144</v>
+        <v>236</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>GRINDER WHEEL SILICON CARBIDE</t>
+          <t>WELDING CABLE 1000 AMPERE</t>
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>3</v>
+        <v>200</v>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Norton</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="E35" s="5" t="n"/>
@@ -3616,19 +2890,19 @@
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
-        <v>145</v>
+        <v>237</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>COTTON ROPE 2MM</t>
+          <t>CABLE LUGS 1000 AMPERE</t>
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>500</v>
+        <v>24</v>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="E36" s="5" t="n"/>
@@ -3636,380 +2910,6 @@
       <c r="G36" s="5" t="n"/>
       <c r="H36" s="4" t="n"/>
     </row>
-    <row r="37">
-      <c r="A37" s="4" t="n">
-        <v>154</v>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>RED OXIDE POWDER</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>Industrial</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="n"/>
-      <c r="F37" s="6" t="n"/>
-      <c r="G37" s="5" t="n"/>
-      <c r="H37" s="4" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="n">
-        <v>159</v>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>CUT PIECES OF CLOTHS FOR CLEANING</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="n"/>
-      <c r="F38" s="6" t="n"/>
-      <c r="G38" s="5" t="n"/>
-      <c r="H38" s="4" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="n">
-        <v>160</v>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>ANCHOR BOLT 10X110</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="n">
-        <v>150</v>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>SMT</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="n"/>
-      <c r="F39" s="6" t="n"/>
-      <c r="G39" s="5" t="n"/>
-      <c r="H39" s="4" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="n">
-        <v>161</v>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>ANCHOR BOLT 12X120</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="n">
-        <v>150</v>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="n"/>
-      <c r="F40" s="6" t="n"/>
-      <c r="G40" s="5" t="n"/>
-      <c r="H40" s="4" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="n">
-        <v>162</v>
-      </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>ANCHOR BOLT 12X160</t>
-        </is>
-      </c>
-      <c r="C41" s="4" t="n">
-        <v>150</v>
-      </c>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="n"/>
-      <c r="F41" s="6" t="n"/>
-      <c r="G41" s="5" t="n"/>
-      <c r="H41" s="4" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="n">
-        <v>164</v>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>WELDING RODS 2.5MM E6013, NO 10 Zodian</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="n">
-        <v>40</v>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>Zodian</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="n"/>
-      <c r="F42" s="6" t="n"/>
-      <c r="G42" s="5" t="n"/>
-      <c r="H42" s="4" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="n">
-        <v>165</v>
-      </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>WELDING RODS 3.25MM E6013 NO 12</t>
-        </is>
-      </c>
-      <c r="C43" s="4" t="n">
-        <v>40</v>
-      </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>Zodian</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="n"/>
-      <c r="F43" s="6" t="n"/>
-      <c r="G43" s="5" t="n"/>
-      <c r="H43" s="4" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="n">
-        <v>166</v>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>WELDING RODS 2.5MM E7018 NO-10</t>
-        </is>
-      </c>
-      <c r="C44" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>Fortrex</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="n"/>
-      <c r="F44" s="6" t="n"/>
-      <c r="G44" s="5" t="n"/>
-      <c r="H44" s="4" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="n">
-        <v>167</v>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>SS WELDING RODS 309L-16 2.6MM NO.12</t>
-        </is>
-      </c>
-      <c r="C45" s="4" t="n">
-        <v>40</v>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>Stainarc</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="n"/>
-      <c r="F45" s="6" t="n"/>
-      <c r="G45" s="5" t="n"/>
-      <c r="H45" s="4" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="n">
-        <v>168</v>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>SS WELDING RODS 316L-16 2.6MM NO.12</t>
-        </is>
-      </c>
-      <c r="C46" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>Stainarc</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="n"/>
-      <c r="F46" s="6" t="n"/>
-      <c r="G46" s="5" t="n"/>
-      <c r="H46" s="4" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="n">
-        <v>177</v>
-      </c>
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>BLIND RIVETS 04MMX25MM (1000PCS)</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>Ingco</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="n"/>
-      <c r="F47" s="6" t="n"/>
-      <c r="G47" s="5" t="n"/>
-      <c r="H47" s="4" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="n">
-        <v>202</v>
-      </c>
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>NEEDLE FILE (5PCS SET)</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="n"/>
-      <c r="F48" s="6" t="n"/>
-      <c r="G48" s="5" t="n"/>
-      <c r="H48" s="4" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="n">
-        <v>230</v>
-      </c>
-      <c r="B49" s="4" t="inlineStr">
-        <is>
-          <t>HYDRAULIC JACK 3 TON</t>
-        </is>
-      </c>
-      <c r="C49" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" s="4" t="inlineStr">
-        <is>
-          <t>Ronix</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="n"/>
-      <c r="F49" s="6" t="n"/>
-      <c r="G49" s="5" t="n"/>
-      <c r="H49" s="4" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="n">
-        <v>234</v>
-      </c>
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>WELDING ELCTRODE HOLDER 1000 AMP</t>
-        </is>
-      </c>
-      <c r="C50" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="n"/>
-      <c r="F50" s="6" t="n"/>
-      <c r="G50" s="5" t="n"/>
-      <c r="H50" s="4" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="n">
-        <v>235</v>
-      </c>
-      <c r="B51" s="4" t="inlineStr">
-        <is>
-          <t>EARTH CLAMP 1000 AMP</t>
-        </is>
-      </c>
-      <c r="C51" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>Industrial</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="n"/>
-      <c r="F51" s="6" t="n"/>
-      <c r="G51" s="5" t="n"/>
-      <c r="H51" s="4" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="4" t="n">
-        <v>236</v>
-      </c>
-      <c r="B52" s="4" t="inlineStr">
-        <is>
-          <t>WELDING CABLE 1000 AMPERE</t>
-        </is>
-      </c>
-      <c r="C52" s="4" t="n">
-        <v>200</v>
-      </c>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>Industrial (copper)</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="n"/>
-      <c r="F52" s="6" t="n"/>
-      <c r="G52" s="5" t="n"/>
-      <c r="H52" s="4" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="4" t="n">
-        <v>237</v>
-      </c>
-      <c r="B53" s="4" t="inlineStr">
-        <is>
-          <t>CABLE LUGS 1000 AMPERE</t>
-        </is>
-      </c>
-      <c r="C53" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="D53" s="4" t="inlineStr">
-        <is>
-          <t>Industrial</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="n"/>
-      <c r="F53" s="6" t="n"/>
-      <c r="G53" s="5" t="n"/>
-      <c r="H53" s="4" t="n"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Verify last 33 items from EU/UK/US listings; all 222 lines now have an online source
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4c5Y1XBRj63SkdBZ73bUS
</commit_message>
<xml_diff>
--- a/quotes/PR-217-228/RFQ_PR217_PR228.xlsx
+++ b/quotes/PR-217-228/RFQ_PR217_PR228.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -560,11 +560,11 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>ALLEN (HEX) KEY 14MM</t>
+          <t>VICE GRIP PLIER 08"</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
@@ -582,15 +582,15 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>ALLEN (HEX) KEY 16MM</t>
+          <t>INTERNAL EXTRACTOR WITH REINFORCED COLLAR</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
@@ -601,182 +601,6 @@
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="5" t="n"/>
       <c r="H7" s="4" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>CIRCLIP PLIER INTERNAL STRAIGHT 230MM</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Licota</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="4" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>CIRCLIP PLIER EXTERNAL STRAIGHT 230MM</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Licota</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="4" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="n">
-        <v>39</v>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>VICE GRIP PLIER 08"</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Licota</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="4" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="n">
-        <v>43</v>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>HEX IMPACT ADAPTOR 1/2" FEMALE TO 1/4" FEMALE</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Licota</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="4" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="n">
-        <v>51</v>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>INTERNAL EXTRACTOR WITH REINFORCED COLLAR</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Licota</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="4" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="n">
-        <v>56</v>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>AIR GREASE GUN 500CC</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Licota</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="6" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="4" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="n">
-        <v>58</v>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>GREASE PIPE 1/4"X12"</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Licota</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="6" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="4" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="n">
-        <v>59</v>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>DOUBLE HANDLE GREASE NOZZLE</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Licota</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -789,7 +613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -860,11 +684,11 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BITS 1/16-1/2" 29 PCS SET</t>
+          <t>HSS DRILL BIT 15.5MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
@@ -872,7 +696,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Dormer A095 (A002 x29)</t>
+          <t>Dormer A130</t>
         </is>
       </c>
       <c r="E5" s="5" t="n"/>
@@ -882,11 +706,11 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 15.5MM TAPER SHANK</t>
+          <t>HSS DRILL BIT 16.5MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
@@ -904,15 +728,15 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 16.5MM TAPER SHANK</t>
+          <t>HSS DRILL BIT 21MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
@@ -926,11 +750,11 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 21MM TAPER SHANK</t>
+          <t>HSS DRILL BIT 30MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
@@ -948,11 +772,11 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 30MM TAPER SHANK</t>
+          <t>HSS DRILL BIT 35MM TAPER SHANK</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
@@ -970,11 +794,11 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>HSS DRILL BIT 35MM TAPER SHANK</t>
+          <t>TAP SET 1/2" BSPF LEFT HAND (Dormer)</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
@@ -982,7 +806,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Dormer A130</t>
+          <t>Dormer</t>
         </is>
       </c>
       <c r="E10" s="5" t="n"/>
@@ -992,11 +816,11 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>TAP SET 1/2" BSPF LEFT HAND (Dormer)</t>
+          <t>TAP SET 3/8" BSPF</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
@@ -1014,11 +838,11 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>99</v>
+        <v>179</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>TAP SET 1/2" BSPF RIGHT HAND</t>
+          <t>TAP SET 1" BSPF LEFT HAND</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
@@ -1036,11 +860,11 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>100</v>
+        <v>181</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>TAP SET 3/8" BSPF</t>
+          <t>TAP SET 1-1/4" BSPF LEFT HAND</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
@@ -1058,11 +882,11 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>TAP SET 1" BSPF LEFT HAND</t>
+          <t>TAP SET 1-1/4" BSPF RIGHT HAND</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
@@ -1080,11 +904,11 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>TAP SET 1" BSPF RIGHT HAND</t>
+          <t>TAP SET M18</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
@@ -1102,15 +926,15 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>181</v>
+        <v>210</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>TAP SET 1-1/4" BSPF LEFT HAND</t>
+          <t>END MILL CUTTER SIZE 18MM</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
@@ -1124,11 +948,11 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>182</v>
+        <v>211</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>TAP SET 1-1/4" BSPF RIGHT HAND</t>
+          <t>END MILL CUTTER SIZE 22MM</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
@@ -1143,94 +967,6 @@
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="5" t="n"/>
       <c r="H17" s="4" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="n">
-        <v>188</v>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>TAP SET M18</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Dormer</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="6" t="n"/>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="4" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="n">
-        <v>210</v>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>END MILL CUTTER SIZE 18MM</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Dormer</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="6" t="n"/>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="4" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="n">
-        <v>211</v>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>END MILL CUTTER SIZE 22MM</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Dormer</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="5" t="n"/>
-      <c r="H20" s="4" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="n">
-        <v>228</v>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>HSS TOOL 16MMX16MMX200MM</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Dormer</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="n"/>
-      <c r="F21" s="6" t="n"/>
-      <c r="G21" s="5" t="n"/>
-      <c r="H21" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1243,7 +979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1314,15 +1050,15 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>ROUNDE FILE 12"</t>
+          <t>ALLEN (HEX) KEY 16MM</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
@@ -1336,19 +1072,19 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>UNIVERSAL PULLER 2-ARMED WITH HOOK BRAKE 21</t>
+          <t>CIRCLIP PLIER INTERNAL STRAIGHT 230MM</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E6" s="5" t="n"/>
@@ -1358,19 +1094,19 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>UNIVERSAL PULLER 2-ARMED 160 X 300 MM 5T</t>
+          <t>CIRCLIP PLIER EXTERNAL STRAIGHT 230MM</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E7" s="5" t="n"/>
@@ -1380,19 +1116,19 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>UNIVERSAL PULLER 2-ARMED 250 X 300 MM 7.5T</t>
+          <t>UNIVERSAL PULLER 2-ARMED WITH HOOK BRAKE 21</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E8" s="5" t="n"/>
@@ -1402,19 +1138,19 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>MANUAL GREASE GUN 5KG</t>
+          <t>UNIVERSAL PULLER 2-ARMED 160 X 300 MM 5T</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E9" s="5" t="n"/>
@@ -1424,15 +1160,15 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>REVOLVING CENTRE MT4</t>
+          <t>UNIVERSAL PULLER 2-ARMED 250 X 300 MM 7.5T</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
@@ -1446,11 +1182,11 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>88</v>
+        <v>55</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>MORSE TAPER EXTENSION SOCKET SLEEVE ADAPT</t>
+          <t>MANUAL GREASE GUN 5KG</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
@@ -1468,19 +1204,19 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>89</v>
+        <v>56</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>MORSE TAPER EXTENSION SOCKET SLEEVE ADAPT</t>
+          <t>AIR GREASE GUN 500CC</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Yato</t>
         </is>
       </c>
       <c r="E12" s="5" t="n"/>
@@ -1490,15 +1226,15 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>90</v>
+        <v>58</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>MORSE TAPER EXTENSION SOCKET SLEEVE ADAPT</t>
+          <t>GREASE PIPE 1/4"X12"</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
@@ -1512,11 +1248,11 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>91</v>
+        <v>66</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>DEAD CENTRE DIAMOND TIP M2</t>
+          <t>REVOLVING CENTRE MT4</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
@@ -1534,11 +1270,11 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>VERNIER DEPTH GUAGE 250MM GRADUATION 0.02M</t>
+          <t>MORSE TAPER EXTENSION SOCKET SLEEVE ADAPT</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
@@ -1546,7 +1282,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Insize</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E15" s="5" t="n"/>
@@ -1556,11 +1292,11 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>CORDLESS DRILL DRIVER 150NM Bosch</t>
+          <t>MORSE TAPER EXTENSION SOCKET SLEEVE ADAPT</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
@@ -1568,7 +1304,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Bosch Professional</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E16" s="5" t="n"/>
@@ -1578,19 +1314,19 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>107</v>
+        <v>90</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>C-CLAMP 12"</t>
+          <t>MORSE TAPER EXTENSION SOCKET SLEEVE ADAPT</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E17" s="5" t="n"/>
@@ -1600,19 +1336,19 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>MAGNET SPIRIT LEVEL 12"</t>
+          <t>DEAD CENTRE DIAMOND TIP M2</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E18" s="5" t="n"/>
@@ -1622,11 +1358,11 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>123</v>
+        <v>96</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>TIG WELDING TORCH AIR-COOLED 5METER</t>
+          <t>VERNIER DEPTH GUAGE 250MM GRADUATION 0.02M</t>
         </is>
       </c>
       <c r="C19" s="4" t="n">
@@ -1634,7 +1370,7 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Insize</t>
         </is>
       </c>
       <c r="E19" s="5" t="n"/>
@@ -1644,19 +1380,19 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>128</v>
+        <v>97</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>CERAMIC CUP NO.6</t>
+          <t>CORDLESS DRILL DRIVER 150NM Bosch</t>
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Bosch Professional</t>
         </is>
       </c>
       <c r="E20" s="5" t="n"/>
@@ -1666,15 +1402,15 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>CERAMIC CUP NO.7</t>
+          <t>TIG WELDING TORCH AIR-COOLED 5METER</t>
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
@@ -1688,15 +1424,15 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>142</v>
+        <v>128</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>GRINDER WHEEL ALUMINIUM OXIDE GRIT 24</t>
+          <t>CERAMIC CUP NO.6</t>
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
@@ -1710,15 +1446,15 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>143</v>
+        <v>129</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>GRINDER WHEEL ALUMINIUM OXIDE GRIT 60</t>
+          <t>CERAMIC CUP NO.7</t>
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
@@ -1732,11 +1468,11 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>GRINDER WHEEL SILICON CARBIDE</t>
+          <t>GRINDER WHEEL ALUMINIUM OXIDE GRIT 24</t>
         </is>
       </c>
       <c r="C24" s="4" t="n">
@@ -1754,15 +1490,15 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>161</v>
+        <v>143</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>ANCHOR BOLT 12X120</t>
+          <t>GRINDER WHEEL ALUMINIUM OXIDE GRIT 60</t>
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>150</v>
+        <v>3</v>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
@@ -1776,15 +1512,15 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>ANCHOR BOLT 12X160</t>
+          <t>GRINDER WHEEL SILICON CARBIDE</t>
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>150</v>
+        <v>3</v>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
@@ -1798,19 +1534,19 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>184</v>
+        <v>161</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>TAP SET M8</t>
+          <t>ANCHOR BOLT 12X120</t>
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>3</v>
+        <v>150</v>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E27" s="5" t="n"/>
@@ -1820,19 +1556,19 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>193</v>
+        <v>162</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>INSIDE CALIPER 20"</t>
+          <t>ANCHOR BOLT 12X160</t>
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Insize</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E28" s="5" t="n"/>
@@ -1842,11 +1578,11 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>OUTSIDE CALIPER 20"</t>
+          <t>INSIDE CALIPER 20"</t>
         </is>
       </c>
       <c r="C29" s="4" t="n">
@@ -1864,11 +1600,11 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>213</v>
+        <v>195</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>DIE NUT SIZE 5MM</t>
+          <t>OUTSIDE CALIPER 20"</t>
         </is>
       </c>
       <c r="C30" s="4" t="n">
@@ -1876,7 +1612,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Insize</t>
         </is>
       </c>
       <c r="E30" s="5" t="n"/>
@@ -1908,11 +1644,11 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>DIE NUT SIZE 8MM</t>
+          <t>DIE NUT SIZE 12MM</t>
         </is>
       </c>
       <c r="C32" s="4" t="n">
@@ -1930,15 +1666,15 @@
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>DIE NUT SIZE 10MM</t>
+          <t>DIE NUT HANDLE SMALL</t>
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
@@ -1952,15 +1688,15 @@
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>DIE NUT SIZE 12MM</t>
+          <t>DIE NUT HANDLE MEDIUM</t>
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
@@ -1974,19 +1710,19 @@
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>DIE NUT HANDLE SMALL</t>
+          <t>BENCH VISE 12"</t>
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E35" s="5" t="n"/>
@@ -1996,19 +1732,19 @@
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>DIE NUT HANDLE MEDIUM</t>
+          <t>HSS TOOL 10MMX10MMX200MM</t>
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E36" s="5" t="n"/>
@@ -2018,19 +1754,19 @@
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>DIE NUT HANDLE LARGE</t>
+          <t>HSS TOOL 12MMX12MMX200MM</t>
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Yato</t>
+          <t>Taiwan</t>
         </is>
       </c>
       <c r="E37" s="5" t="n"/>
@@ -2040,15 +1776,15 @@
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>BENCH VISE 12"</t>
+          <t>HSS TOOL 16MMX16MMX200MM</t>
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
@@ -2062,11 +1798,11 @@
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>HSS TOOL 10MMX10MMX200MM</t>
+          <t>HSS PARTING OFF TOOL 1/8" X 3/4" X 8"</t>
         </is>
       </c>
       <c r="C39" s="4" t="n">
@@ -2081,50 +1817,6 @@
       <c r="F39" s="6" t="n"/>
       <c r="G39" s="5" t="n"/>
       <c r="H39" s="4" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="n">
-        <v>227</v>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>HSS TOOL 12MMX12MMX200MM</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>Taiwan</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="n"/>
-      <c r="F40" s="6" t="n"/>
-      <c r="G40" s="5" t="n"/>
-      <c r="H40" s="4" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="n">
-        <v>229</v>
-      </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>HSS PARTING OFF TOOL 1/8" X 3/4" X 8"</t>
-        </is>
-      </c>
-      <c r="C41" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>Taiwan</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="n"/>
-      <c r="F41" s="6" t="n"/>
-      <c r="G41" s="5" t="n"/>
-      <c r="H41" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2137,7 +1829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2450,19 +2142,19 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>CYLINDER KEY/SPANNER</t>
+          <t>AC/DC SINGLE PHASE WELDING PLANT 300 AMP</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>WACTA20</t>
         </is>
       </c>
       <c r="E16" s="5" t="n"/>
@@ -2472,19 +2164,19 @@
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>AC/DC SINGLE PHASE WELDING PLANT 300 AMP</t>
+          <t>ARGON GAS HOSE 06MM</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>WACTA20</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="E17" s="5" t="n"/>
@@ -2494,15 +2186,15 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>124</v>
+        <v>154</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>TORCH HEAD ARGON WELDING</t>
+          <t>RED OXIDE POWDER</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
@@ -2516,19 +2208,19 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>132</v>
+        <v>159</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>ARGON GAS HOSE 06MM</t>
+          <t>CUT PIECES OF CLOTHS FOR CLEANING</t>
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Local</t>
         </is>
       </c>
       <c r="E19" s="5" t="n"/>
@@ -2538,19 +2230,19 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>BUFFING DISC 125MM</t>
+          <t>ANCHOR BOLT 10X110</t>
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>24</v>
+        <v>150</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>SMT</t>
         </is>
       </c>
       <c r="E20" s="5" t="n"/>
@@ -2560,19 +2252,19 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>145</v>
+        <v>164</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>COTTON ROPE 2MM</t>
+          <t>WELDING RODS 2.5MM E6013, NO 10 Zodian</t>
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>500</v>
+        <v>40</v>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Zodian</t>
         </is>
       </c>
       <c r="E21" s="5" t="n"/>
@@ -2582,19 +2274,19 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>154</v>
+        <v>165</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>RED OXIDE POWDER</t>
+          <t>WELDING RODS 3.25MM E6013 NO 12</t>
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Zodian</t>
         </is>
       </c>
       <c r="E22" s="5" t="n"/>
@@ -2604,19 +2296,19 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>CUT PIECES OF CLOTHS FOR CLEANING</t>
+          <t>WELDING RODS 2.5MM E7018 NO-10</t>
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Fortrex</t>
         </is>
       </c>
       <c r="E23" s="5" t="n"/>
@@ -2626,19 +2318,19 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>ANCHOR BOLT 10X110</t>
+          <t>SS WELDING RODS 309L-16 2.6MM NO.12</t>
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>150</v>
+        <v>40</v>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>SMT</t>
+          <t>Stainarc</t>
         </is>
       </c>
       <c r="E24" s="5" t="n"/>
@@ -2648,19 +2340,19 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>WELDING RODS 2.5MM E6013, NO 10 Zodian</t>
+          <t>SS WELDING RODS 316L-16 2.6MM NO.12</t>
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Zodian</t>
+          <t>Stainarc</t>
         </is>
       </c>
       <c r="E25" s="5" t="n"/>
@@ -2670,19 +2362,19 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>WELDING RODS 3.25MM E6013 NO 12</t>
+          <t>BLIND RIVETS 04MMX25MM (1000PCS)</t>
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Zodian</t>
+          <t>Generic</t>
         </is>
       </c>
       <c r="E26" s="5" t="n"/>
@@ -2692,19 +2384,19 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>166</v>
+        <v>202</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>WELDING RODS 2.5MM E7018 NO-10</t>
+          <t>NEEDLE FILE (5PCS SET)</t>
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Fortrex</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E27" s="5" t="n"/>
@@ -2714,19 +2406,19 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>167</v>
+        <v>230</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>SS WELDING RODS 309L-16 2.6MM NO.12</t>
+          <t>HYDRAULIC JACK 3 TON</t>
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Stainarc</t>
+          <t>Ronix</t>
         </is>
       </c>
       <c r="E28" s="5" t="n"/>
@@ -2736,19 +2428,19 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>168</v>
+        <v>234</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>SS WELDING RODS 316L-16 2.6MM NO.12</t>
+          <t>WELDING ELCTRODE HOLDER 1000 AMP</t>
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Stainarc</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E29" s="5" t="n"/>
@@ -2758,11 +2450,11 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>177</v>
+        <v>235</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>BLIND RIVETS 04MMX25MM (1000PCS)</t>
+          <t>EARTH CLAMP 1000 AMP</t>
         </is>
       </c>
       <c r="C30" s="4" t="n">
@@ -2770,7 +2462,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Generic</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="E30" s="5" t="n"/>
@@ -2780,19 +2472,19 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>202</v>
+        <v>236</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>NEEDLE FILE (5PCS SET)</t>
+          <t>WELDING CABLE 1000 AMPERE</t>
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="E31" s="5" t="n"/>
@@ -2802,19 +2494,19 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>HYDRAULIC JACK 3 TON</t>
+          <t>CABLE LUGS 1000 AMPERE</t>
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Ronix</t>
+          <t>Industrial</t>
         </is>
       </c>
       <c r="E32" s="5" t="n"/>
@@ -2822,94 +2514,6 @@
       <c r="G32" s="5" t="n"/>
       <c r="H32" s="4" t="n"/>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="n">
-        <v>234</v>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>WELDING ELCTRODE HOLDER 1000 AMP</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="n"/>
-      <c r="F33" s="6" t="n"/>
-      <c r="G33" s="5" t="n"/>
-      <c r="H33" s="4" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="n">
-        <v>235</v>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>EARTH CLAMP 1000 AMP</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>Industrial</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="n"/>
-      <c r="F34" s="6" t="n"/>
-      <c r="G34" s="5" t="n"/>
-      <c r="H34" s="4" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="n">
-        <v>236</v>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>WELDING CABLE 1000 AMPERE</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="n">
-        <v>200</v>
-      </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>Industrial</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="n"/>
-      <c r="F35" s="6" t="n"/>
-      <c r="G35" s="5" t="n"/>
-      <c r="H35" s="4" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="n">
-        <v>237</v>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>CABLE LUGS 1000 AMPERE</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>Industrial</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="n"/>
-      <c r="F36" s="6" t="n"/>
-      <c r="G36" s="5" t="n"/>
-      <c r="H36" s="4" t="n"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>